<commit_message>
adding more systems for app to pull from
</commit_message>
<xml_diff>
--- a/backend/assets/data/fujitsu_capacities_calculated.xlsx
+++ b/backend/assets/data/fujitsu_capacities_calculated.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29609"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
@@ -16,7 +16,7 @@
     <sheet name="indoor_combinations" sheetId="2" r:id="rId1"/>
     <sheet name="capacity_70_0" sheetId="1" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -39,28 +39,10 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="413" uniqueCount="21">
   <si>
-    <t>Indoor Capacity (kBtu/h)</t>
-  </si>
-  <si>
-    <t>Outdoor Temp (°F)</t>
-  </si>
-  <si>
-    <t>Capacity at 70F (Btu/h)</t>
-  </si>
-  <si>
-    <t>AOUH24KWAH3</t>
-  </si>
-  <si>
-    <t>AOUH18KWAH2</t>
-  </si>
-  <si>
     <t>Model</t>
   </si>
   <si>
-    <t>AOUH36KWAH4</t>
-  </si>
-  <si>
-    <t>Capacity at 70°F Indoor / 0°F Outdoor</t>
+    <t>Type</t>
   </si>
   <si>
     <t>Indoor Capacity</t>
@@ -72,13 +54,28 @@
     <t>Unit 2</t>
   </si>
   <si>
+    <t>Unit 3</t>
+  </si>
+  <si>
+    <t>Unit 4</t>
+  </si>
+  <si>
     <t>Max Capacity Unit 1</t>
   </si>
   <si>
     <t>Max Capacity Unit 2</t>
   </si>
   <si>
+    <t>Max Capacity Unit 3</t>
+  </si>
+  <si>
+    <t>Max Capacity Unit 4</t>
+  </si>
+  <si>
     <t>Total Capacity</t>
+  </si>
+  <si>
+    <t>AOUH18KWAH2</t>
   </si>
   <si>
     <t>Non-ducted</t>
@@ -87,26 +84,29 @@
     <t>Ducted</t>
   </si>
   <si>
-    <t>Unit 3</t>
+    <t>AOUH24KWAH3</t>
   </si>
   <si>
-    <t>Max Capacity Unit 3</t>
+    <t>AOUH36KWAH4</t>
   </si>
   <si>
-    <t>Unit 4</t>
+    <t>Capacity at 70°F Indoor / 0°F Outdoor</t>
   </si>
   <si>
-    <t>Max Capacity Unit 4</t>
+    <t>Indoor Capacity (kBtu/h)</t>
   </si>
   <si>
-    <t>Type</t>
+    <t>Outdoor Temp (°F)</t>
+  </si>
+  <si>
+    <t>Capacity at 70F (Btu/h)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -428,62 +428,62 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2E4304B4-14C5-40DF-85A6-AED3FDED911B}">
   <dimension ref="A1:N177"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.45"/>
   <cols>
-    <col min="1" max="1" width="14.26953125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.6328125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="14" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="5.7265625" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="5.7265625" customWidth="1"/>
-    <col min="8" max="9" width="17.453125" bestFit="1" customWidth="1"/>
-    <col min="10" max="11" width="17.453125" customWidth="1"/>
-    <col min="12" max="12" width="12.453125" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="5.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="5.7109375" customWidth="1"/>
+    <col min="8" max="9" width="17.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="11" width="17.42578125" customWidth="1"/>
+    <col min="12" max="12" width="12.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:14">
       <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="B1" t="s">
-        <v>20</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="D1" t="s">
-        <v>9</v>
-      </c>
-      <c r="E1" t="s">
+      <c r="J1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="F1" t="s">
-        <v>16</v>
-      </c>
-      <c r="G1" t="s">
-        <v>18</v>
-      </c>
-      <c r="H1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="I1" t="s">
-        <v>12</v>
-      </c>
-      <c r="J1" t="s">
-        <v>17</v>
-      </c>
-      <c r="K1" t="s">
-        <v>19</v>
-      </c>
-      <c r="L1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.35">
+    </row>
+    <row r="2" spans="1:14">
       <c r="A2" t="s">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="B2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C2">
         <v>14</v>
@@ -504,12 +504,12 @@
         <v>16335</v>
       </c>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:14">
       <c r="A3" t="s">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="B3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C3">
         <v>16</v>
@@ -530,12 +530,12 @@
         <v>17750</v>
       </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:14">
       <c r="A4" t="s">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="B4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C4">
         <v>19</v>
@@ -556,12 +556,12 @@
         <v>19725</v>
       </c>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:14">
       <c r="A5" t="s">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="B5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C5">
         <v>22</v>
@@ -582,12 +582,12 @@
         <v>19725</v>
       </c>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:14">
       <c r="A6" t="s">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="B6" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C6">
         <v>18</v>
@@ -608,12 +608,12 @@
         <v>19725</v>
       </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:14">
       <c r="A7" t="s">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="B7" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C7">
         <v>21</v>
@@ -634,12 +634,12 @@
         <v>19725</v>
       </c>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:14">
       <c r="A8" t="s">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="B8" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C8">
         <v>24</v>
@@ -660,12 +660,12 @@
         <v>19725</v>
       </c>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:14">
       <c r="A9" t="s">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="B9" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C9">
         <v>24</v>
@@ -686,12 +686,12 @@
         <v>19725</v>
       </c>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:14">
       <c r="A10" t="s">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="B10" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C10">
         <v>14</v>
@@ -712,12 +712,12 @@
         <v>16335</v>
       </c>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:14">
       <c r="A11" t="s">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="B11" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C11">
         <v>16</v>
@@ -738,12 +738,12 @@
         <v>17750</v>
       </c>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:14">
       <c r="A12" t="s">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="B12" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C12">
         <v>19</v>
@@ -764,12 +764,12 @@
         <v>19725</v>
       </c>
     </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:14">
       <c r="A13" t="s">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C13">
         <v>18</v>
@@ -790,12 +790,12 @@
         <v>19725</v>
       </c>
     </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:14">
       <c r="A14" t="s">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="B14" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C14">
         <v>21</v>
@@ -816,12 +816,12 @@
         <v>19725</v>
       </c>
     </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:14">
       <c r="A15" t="s">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="B15" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C15">
         <v>24</v>
@@ -842,12 +842,12 @@
         <v>19725</v>
       </c>
     </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:14">
       <c r="A16" t="s">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C16">
         <v>14</v>
@@ -872,12 +872,12 @@
       <c r="M16" s="1"/>
       <c r="N16" s="1"/>
     </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:14">
       <c r="A17" t="s">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="B17" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C17">
         <v>16</v>
@@ -902,12 +902,12 @@
       <c r="M17" s="1"/>
       <c r="N17" s="1"/>
     </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:14">
       <c r="A18" t="s">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="B18" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C18">
         <v>19</v>
@@ -932,12 +932,12 @@
       <c r="M18" s="1"/>
       <c r="N18" s="1"/>
     </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:14">
       <c r="A19" t="s">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="B19" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C19">
         <v>22</v>
@@ -962,12 +962,12 @@
       <c r="M19" s="1"/>
       <c r="N19" s="1"/>
     </row>
-    <row r="20" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:14">
       <c r="A20" t="s">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="B20" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C20">
         <v>25</v>
@@ -992,12 +992,12 @@
       <c r="M20" s="1"/>
       <c r="N20" s="1"/>
     </row>
-    <row r="21" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:14">
       <c r="A21" t="s">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="B21" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C21">
         <v>18</v>
@@ -1022,12 +1022,12 @@
       <c r="M21" s="1"/>
       <c r="N21" s="1"/>
     </row>
-    <row r="22" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:14">
       <c r="A22" t="s">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="B22" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C22">
         <v>21</v>
@@ -1052,12 +1052,12 @@
       <c r="M22" s="1"/>
       <c r="N22" s="1"/>
     </row>
-    <row r="23" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:14">
       <c r="A23" t="s">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="B23" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C23">
         <v>24</v>
@@ -1082,12 +1082,12 @@
       <c r="M23" s="1"/>
       <c r="N23" s="1"/>
     </row>
-    <row r="24" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:14">
       <c r="A24" t="s">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="B24" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C24">
         <v>27</v>
@@ -1112,12 +1112,12 @@
       <c r="M24" s="1"/>
       <c r="N24" s="1"/>
     </row>
-    <row r="25" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:14">
       <c r="A25" t="s">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="B25" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C25">
         <v>24</v>
@@ -1142,12 +1142,12 @@
       <c r="M25" s="1"/>
       <c r="N25" s="1"/>
     </row>
-    <row r="26" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:14">
       <c r="A26" t="s">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="B26" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C26">
         <v>27</v>
@@ -1172,12 +1172,12 @@
       <c r="M26" s="1"/>
       <c r="N26" s="1"/>
     </row>
-    <row r="27" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:14">
       <c r="A27" t="s">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="B27" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C27">
         <v>30</v>
@@ -1202,12 +1202,12 @@
       <c r="M27" s="1"/>
       <c r="N27" s="1"/>
     </row>
-    <row r="28" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:14">
       <c r="A28" t="s">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="B28" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C28">
         <v>30</v>
@@ -1232,12 +1232,12 @@
       <c r="M28" s="1"/>
       <c r="N28" s="1"/>
     </row>
-    <row r="29" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:14">
       <c r="A29" t="s">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="B29" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C29">
         <v>21</v>
@@ -1267,12 +1267,12 @@
       <c r="M29" s="1"/>
       <c r="N29" s="1"/>
     </row>
-    <row r="30" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:14">
       <c r="A30" t="s">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="B30" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C30">
         <v>23</v>
@@ -1302,12 +1302,12 @@
       <c r="M30" s="1"/>
       <c r="N30" s="1"/>
     </row>
-    <row r="31" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:14">
       <c r="A31" t="s">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="B31" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C31">
         <v>26</v>
@@ -1337,12 +1337,12 @@
       <c r="M31" s="1"/>
       <c r="N31" s="1"/>
     </row>
-    <row r="32" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:14">
       <c r="A32" t="s">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="B32" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C32">
         <v>29</v>
@@ -1372,12 +1372,12 @@
       <c r="M32" s="1"/>
       <c r="N32" s="1"/>
     </row>
-    <row r="33" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:14">
       <c r="A33" t="s">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="B33" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C33">
         <v>25</v>
@@ -1407,12 +1407,12 @@
       <c r="M33" s="1"/>
       <c r="N33" s="1"/>
     </row>
-    <row r="34" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:14">
       <c r="A34" t="s">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="B34" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C34">
         <v>28</v>
@@ -1442,12 +1442,12 @@
       <c r="M34" s="1"/>
       <c r="N34" s="1"/>
     </row>
-    <row r="35" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:14">
       <c r="A35" t="s">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="B35" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C35">
         <v>31</v>
@@ -1477,12 +1477,12 @@
       <c r="M35" s="1"/>
       <c r="N35" s="1"/>
     </row>
-    <row r="36" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:14">
       <c r="A36" t="s">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="B36" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C36">
         <v>31</v>
@@ -1512,12 +1512,12 @@
       <c r="M36" s="1"/>
       <c r="N36" s="1"/>
     </row>
-    <row r="37" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:14">
       <c r="A37" t="s">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="B37" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C37">
         <v>27</v>
@@ -1547,12 +1547,12 @@
       <c r="M37" s="1"/>
       <c r="N37" s="1"/>
     </row>
-    <row r="38" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:14">
       <c r="A38" t="s">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="B38" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C38">
         <v>30</v>
@@ -1582,12 +1582,12 @@
       <c r="M38" s="1"/>
       <c r="N38" s="1"/>
     </row>
-    <row r="39" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:14">
       <c r="A39" t="s">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="B39" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C39">
         <v>14</v>
@@ -1610,12 +1610,12 @@
         <v>16115</v>
       </c>
     </row>
-    <row r="40" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:14">
       <c r="A40" t="s">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="B40" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C40">
         <v>16</v>
@@ -1638,12 +1638,12 @@
         <v>17785</v>
       </c>
     </row>
-    <row r="41" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:14">
       <c r="A41" t="s">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="B41" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C41">
         <v>19</v>
@@ -1666,12 +1666,12 @@
         <v>19165</v>
       </c>
     </row>
-    <row r="42" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:14">
       <c r="A42" t="s">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="B42" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C42">
         <v>25</v>
@@ -1694,12 +1694,12 @@
         <v>22505</v>
       </c>
     </row>
-    <row r="43" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:14">
       <c r="A43" t="s">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="B43" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C43">
         <v>18</v>
@@ -1722,12 +1722,12 @@
         <v>18440</v>
       </c>
     </row>
-    <row r="44" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:14">
       <c r="A44" t="s">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="B44" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C44">
         <v>21</v>
@@ -1750,12 +1750,12 @@
         <v>20690</v>
       </c>
     </row>
-    <row r="45" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:14">
       <c r="A45" t="s">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="B45" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C45">
         <v>27</v>
@@ -1778,12 +1778,12 @@
         <v>22505</v>
       </c>
     </row>
-    <row r="46" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:14">
       <c r="A46" t="s">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="B46" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C46">
         <v>24</v>
@@ -1806,12 +1806,12 @@
         <v>22505</v>
       </c>
     </row>
-    <row r="47" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:14">
       <c r="A47" t="s">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="B47" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C47">
         <v>30</v>
@@ -1834,12 +1834,12 @@
         <v>22505</v>
       </c>
     </row>
-    <row r="48" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:14">
       <c r="A48" t="s">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="B48" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C48">
         <v>21</v>
@@ -1868,12 +1868,12 @@
         <v>20690</v>
       </c>
     </row>
-    <row r="49" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:12">
       <c r="A49" t="s">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="B49" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C49">
         <v>23</v>
@@ -1902,12 +1902,12 @@
         <v>22505</v>
       </c>
     </row>
-    <row r="50" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:12">
       <c r="A50" t="s">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="B50" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C50">
         <v>26</v>
@@ -1936,12 +1936,12 @@
         <v>22505</v>
       </c>
     </row>
-    <row r="51" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:12">
       <c r="A51" t="s">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="B51" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C51">
         <v>25</v>
@@ -1970,12 +1970,12 @@
         <v>22505</v>
       </c>
     </row>
-    <row r="52" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:12">
       <c r="A52" t="s">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="B52" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C52">
         <v>28</v>
@@ -2004,12 +2004,12 @@
         <v>22505</v>
       </c>
     </row>
-    <row r="53" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:12">
       <c r="A53" t="s">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="B53" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C53">
         <v>31</v>
@@ -2038,12 +2038,12 @@
         <v>22505</v>
       </c>
     </row>
-    <row r="54" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:12">
       <c r="A54" t="s">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="B54" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C54">
         <v>27</v>
@@ -2072,12 +2072,12 @@
         <v>22505</v>
       </c>
     </row>
-    <row r="55" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:12">
       <c r="A55" t="s">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="B55" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C55">
         <v>30</v>
@@ -2106,12 +2106,12 @@
         <v>22505</v>
       </c>
     </row>
-    <row r="56" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:12">
       <c r="A56" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B56" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C56">
         <v>31</v>
@@ -2132,12 +2132,12 @@
         <v>27260</v>
       </c>
     </row>
-    <row r="57" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:12">
       <c r="A57" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B57" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C57">
         <v>33</v>
@@ -2158,12 +2158,12 @@
         <v>28560</v>
       </c>
     </row>
-    <row r="58" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:12">
       <c r="A58" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B58" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C58">
         <v>30</v>
@@ -2184,12 +2184,12 @@
         <v>26610</v>
       </c>
     </row>
-    <row r="59" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:12">
       <c r="A59" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B59" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C59">
         <v>36</v>
@@ -2210,12 +2210,12 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="60" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:12">
       <c r="A60" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B60" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C60">
         <v>33</v>
@@ -2236,12 +2236,12 @@
         <v>28560</v>
       </c>
     </row>
-    <row r="61" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:12">
       <c r="A61" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B61" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C61">
         <v>39</v>
@@ -2262,12 +2262,12 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="62" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:12">
       <c r="A62" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B62" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C62">
         <v>36</v>
@@ -2288,12 +2288,12 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="63" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:12">
       <c r="A63" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B63" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C63">
         <v>42</v>
@@ -2314,12 +2314,12 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="64" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:12">
       <c r="A64" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B64" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C64">
         <v>26</v>
@@ -2346,12 +2346,12 @@
         <v>24010</v>
       </c>
     </row>
-    <row r="65" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:12">
       <c r="A65" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B65" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C65">
         <v>29</v>
@@ -2378,12 +2378,12 @@
         <v>25960</v>
       </c>
     </row>
-    <row r="66" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:12">
       <c r="A66" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B66" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C66">
         <v>32</v>
@@ -2410,12 +2410,12 @@
         <v>27910</v>
       </c>
     </row>
-    <row r="67" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:12">
       <c r="A67" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B67" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C67">
         <v>38</v>
@@ -2442,12 +2442,12 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="68" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:12">
       <c r="A68" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B68" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C68">
         <v>25</v>
@@ -2474,12 +2474,12 @@
         <v>23360</v>
       </c>
     </row>
-    <row r="69" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:12">
       <c r="A69" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B69" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C69">
         <v>28</v>
@@ -2506,12 +2506,12 @@
         <v>25310</v>
       </c>
     </row>
-    <row r="70" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:12">
       <c r="A70" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B70" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C70">
         <v>31</v>
@@ -2538,12 +2538,12 @@
         <v>27260</v>
       </c>
     </row>
-    <row r="71" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:12">
       <c r="A71" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B71" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C71">
         <v>34</v>
@@ -2570,12 +2570,12 @@
         <v>29260</v>
       </c>
     </row>
-    <row r="72" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:12">
       <c r="A72" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B72" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C72">
         <v>40</v>
@@ -2602,12 +2602,12 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="73" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:12">
       <c r="A73" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B73" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C73">
         <v>31</v>
@@ -2634,12 +2634,12 @@
         <v>27260</v>
       </c>
     </row>
-    <row r="74" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:12">
       <c r="A74" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B74" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C74">
         <v>34</v>
@@ -2666,12 +2666,12 @@
         <v>29260</v>
       </c>
     </row>
-    <row r="75" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:12">
       <c r="A75" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B75" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C75">
         <v>37</v>
@@ -2698,12 +2698,12 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="76" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:12">
       <c r="A76" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B76" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C76">
         <v>43</v>
@@ -2730,12 +2730,12 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="77" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:12">
       <c r="A77" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B77" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C77">
         <v>37</v>
@@ -2762,12 +2762,12 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="78" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:12">
       <c r="A78" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B78" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C78">
         <v>40</v>
@@ -2794,12 +2794,12 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="79" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:12">
       <c r="A79" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B79" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C79">
         <v>46</v>
@@ -2826,12 +2826,12 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="80" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:12">
       <c r="A80" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B80" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C80">
         <v>43</v>
@@ -2858,12 +2858,12 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="81" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:12">
       <c r="A81" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B81" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C81">
         <v>27</v>
@@ -2890,12 +2890,12 @@
         <v>24660</v>
       </c>
     </row>
-    <row r="82" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:12">
       <c r="A82" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B82" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C82">
         <v>30</v>
@@ -2922,12 +2922,12 @@
         <v>26610</v>
       </c>
     </row>
-    <row r="83" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:12">
       <c r="A83" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B83" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C83">
         <v>33</v>
@@ -2954,12 +2954,12 @@
         <v>28560</v>
       </c>
     </row>
-    <row r="84" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:12">
       <c r="A84" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B84" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C84">
         <v>36</v>
@@ -2986,12 +2986,12 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="85" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:12">
       <c r="A85" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B85" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C85">
         <v>42</v>
@@ -3018,12 +3018,12 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="86" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:12">
       <c r="A86" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B86" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C86">
         <v>33</v>
@@ -3050,12 +3050,12 @@
         <v>28560</v>
       </c>
     </row>
-    <row r="87" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:12">
       <c r="A87" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B87" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C87">
         <v>36</v>
@@ -3082,12 +3082,12 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="88" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:12">
       <c r="A88" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B88" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C88">
         <v>39</v>
@@ -3114,12 +3114,12 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="89" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:12">
       <c r="A89" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B89" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C89">
         <v>45</v>
@@ -3146,12 +3146,12 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="90" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:12">
       <c r="A90" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B90" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C90">
         <v>39</v>
@@ -3178,12 +3178,12 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="91" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:12">
       <c r="A91" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B91" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C91">
         <v>42</v>
@@ -3210,12 +3210,12 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="92" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:12">
       <c r="A92" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B92" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C92">
         <v>45</v>
@@ -3242,12 +3242,12 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="93" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:12">
       <c r="A93" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B93" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C93">
         <v>36</v>
@@ -3274,12 +3274,12 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="94" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:12">
       <c r="A94" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B94" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C94">
         <v>39</v>
@@ -3306,12 +3306,12 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="95" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:12">
       <c r="A95" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B95" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C95">
         <v>42</v>
@@ -3338,12 +3338,12 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="96" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:12">
       <c r="A96" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B96" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C96">
         <v>42</v>
@@ -3370,12 +3370,12 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="97" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:12">
       <c r="A97" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B97" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C97">
         <v>45</v>
@@ -3402,12 +3402,12 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="98" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:12">
       <c r="A98" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B98" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C98">
         <v>45</v>
@@ -3434,12 +3434,12 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="99" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:12">
       <c r="A99" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B99" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C99">
         <v>28</v>
@@ -3472,12 +3472,12 @@
         <v>25310</v>
       </c>
     </row>
-    <row r="100" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:12">
       <c r="A100" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B100" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C100">
         <v>30</v>
@@ -3510,12 +3510,12 @@
         <v>26610</v>
       </c>
     </row>
-    <row r="101" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:12">
       <c r="A101" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B101" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C101">
         <v>33</v>
@@ -3548,12 +3548,12 @@
         <v>28560</v>
       </c>
     </row>
-    <row r="102" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:12">
       <c r="A102" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B102" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C102">
         <v>36</v>
@@ -3586,12 +3586,12 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="103" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:12">
       <c r="A103" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B103" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C103">
         <v>39</v>
@@ -3624,12 +3624,12 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="104" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:12">
       <c r="A104" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B104" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C104">
         <v>45</v>
@@ -3662,12 +3662,12 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="105" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:12">
       <c r="A105" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B105" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C105">
         <v>32</v>
@@ -3700,12 +3700,12 @@
         <v>27910</v>
       </c>
     </row>
-    <row r="106" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:12">
       <c r="A106" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B106" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C106">
         <v>35</v>
@@ -3738,12 +3738,12 @@
         <v>29880</v>
       </c>
     </row>
-    <row r="107" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:12">
       <c r="A107" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B107" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C107">
         <v>38</v>
@@ -3776,12 +3776,12 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="108" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:12">
       <c r="A108" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B108" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C108">
         <v>41</v>
@@ -3814,12 +3814,12 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="109" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:12">
       <c r="A109" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B109" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C109">
         <v>38</v>
@@ -3852,12 +3852,12 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="110" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:12">
       <c r="A110" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B110" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C110">
         <v>41</v>
@@ -3890,12 +3890,12 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="111" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:12">
       <c r="A111" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B111" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C111">
         <v>44</v>
@@ -3928,12 +3928,12 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="112" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:12">
       <c r="A112" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B112" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C112">
         <v>44</v>
@@ -3966,12 +3966,12 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="113" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:12">
       <c r="A113" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B113" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C113">
         <v>34</v>
@@ -4004,12 +4004,12 @@
         <v>29260</v>
       </c>
     </row>
-    <row r="114" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:12">
       <c r="A114" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B114" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C114">
         <v>37</v>
@@ -4042,12 +4042,12 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="115" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:12">
       <c r="A115" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B115" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C115">
         <v>40</v>
@@ -4080,12 +4080,12 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="116" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:12">
       <c r="A116" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B116" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C116">
         <v>43</v>
@@ -4118,12 +4118,12 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="117" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:12">
       <c r="A117" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B117" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C117">
         <v>40</v>
@@ -4156,12 +4156,12 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="118" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:12">
       <c r="A118" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B118" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C118">
         <v>43</v>
@@ -4194,12 +4194,12 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="119" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:12">
       <c r="A119" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B119" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C119">
         <v>46</v>
@@ -4232,12 +4232,12 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="120" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:12">
       <c r="A120" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B120" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C120">
         <v>46</v>
@@ -4270,12 +4270,12 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="121" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:12">
       <c r="A121" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B121" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C121">
         <v>43</v>
@@ -4308,12 +4308,12 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="122" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:12">
       <c r="A122" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B122" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C122">
         <v>46</v>
@@ -4346,12 +4346,12 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="123" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:12">
       <c r="A123" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B123" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C123">
         <v>36</v>
@@ -4384,12 +4384,12 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="124" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:12">
       <c r="A124" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B124" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C124">
         <v>39</v>
@@ -4422,12 +4422,12 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="125" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:12">
       <c r="A125" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B125" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C125">
         <v>42</v>
@@ -4460,12 +4460,12 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="126" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:12">
       <c r="A126" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B126" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C126">
         <v>45</v>
@@ -4498,12 +4498,12 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="127" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:12">
       <c r="A127" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B127" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C127">
         <v>42</v>
@@ -4536,12 +4536,12 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="128" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:12">
       <c r="A128" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B128" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C128">
         <v>45</v>
@@ -4574,12 +4574,12 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="129" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:12">
       <c r="A129" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B129" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C129">
         <v>45</v>
@@ -4612,12 +4612,12 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="130" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:12">
       <c r="A130" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B130" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C130">
         <v>31</v>
@@ -4638,12 +4638,12 @@
         <v>27260</v>
       </c>
     </row>
-    <row r="131" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:12">
       <c r="A131" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B131" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C131">
         <v>33</v>
@@ -4664,12 +4664,12 @@
         <v>28560</v>
       </c>
     </row>
-    <row r="132" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:12">
       <c r="A132" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B132" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C132">
         <v>30</v>
@@ -4690,12 +4690,12 @@
         <v>26610</v>
       </c>
     </row>
-    <row r="133" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:12">
       <c r="A133" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B133" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C133">
         <v>36</v>
@@ -4716,12 +4716,12 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="134" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:12">
       <c r="A134" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B134" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C134">
         <v>36</v>
@@ -4742,12 +4742,12 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="135" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:12">
       <c r="A135" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B135" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C135">
         <v>42</v>
@@ -4768,12 +4768,12 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="136" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:12">
       <c r="A136" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B136" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C136">
         <v>26</v>
@@ -4800,12 +4800,12 @@
         <v>24010</v>
       </c>
     </row>
-    <row r="137" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:12">
       <c r="A137" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B137" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C137">
         <v>32</v>
@@ -4832,12 +4832,12 @@
         <v>27910</v>
       </c>
     </row>
-    <row r="138" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:12">
       <c r="A138" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B138" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C138">
         <v>38</v>
@@ -4864,12 +4864,12 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="139" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:12">
       <c r="A139" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B139" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C139">
         <v>25</v>
@@ -4896,12 +4896,12 @@
         <v>23360</v>
       </c>
     </row>
-    <row r="140" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:12">
       <c r="A140" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B140" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C140">
         <v>28</v>
@@ -4928,12 +4928,12 @@
         <v>25310</v>
       </c>
     </row>
-    <row r="141" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:12">
       <c r="A141" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B141" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C141">
         <v>34</v>
@@ -4960,12 +4960,12 @@
         <v>29260</v>
       </c>
     </row>
-    <row r="142" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:12">
       <c r="A142" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B142" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C142">
         <v>40</v>
@@ -4992,12 +4992,12 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="143" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:12">
       <c r="A143" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B143" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C143">
         <v>31</v>
@@ -5024,12 +5024,12 @@
         <v>27260</v>
       </c>
     </row>
-    <row r="144" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:12">
       <c r="A144" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B144" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C144">
         <v>37</v>
@@ -5056,12 +5056,12 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="145" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:12">
       <c r="A145" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B145" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C145">
         <v>43</v>
@@ -5088,12 +5088,12 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="146" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:12">
       <c r="A146" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B146" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C146">
         <v>43</v>
@@ -5120,12 +5120,12 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="147" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:12">
       <c r="A147" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B147" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C147">
         <v>27</v>
@@ -5152,12 +5152,12 @@
         <v>24660</v>
       </c>
     </row>
-    <row r="148" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:12">
       <c r="A148" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B148" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C148">
         <v>30</v>
@@ -5184,12 +5184,12 @@
         <v>26610</v>
       </c>
     </row>
-    <row r="149" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:12">
       <c r="A149" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B149" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C149">
         <v>36</v>
@@ -5216,12 +5216,12 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="150" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:12">
       <c r="A150" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B150" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C150">
         <v>42</v>
@@ -5248,12 +5248,12 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="151" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:12">
       <c r="A151" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B151" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C151">
         <v>33</v>
@@ -5280,12 +5280,12 @@
         <v>28560</v>
       </c>
     </row>
-    <row r="152" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:12">
       <c r="A152" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B152" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C152">
         <v>39</v>
@@ -5312,12 +5312,12 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="153" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:12">
       <c r="A153" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B153" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C153">
         <v>45</v>
@@ -5344,12 +5344,12 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="154" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:12">
       <c r="A154" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B154" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C154">
         <v>45</v>
@@ -5376,12 +5376,12 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="155" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:12">
       <c r="A155" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B155" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C155">
         <v>36</v>
@@ -5408,12 +5408,12 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="156" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:12">
       <c r="A156" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B156" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C156">
         <v>42</v>
@@ -5440,12 +5440,12 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="157" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:12">
       <c r="A157" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B157" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C157">
         <v>28</v>
@@ -5478,12 +5478,12 @@
         <v>25310</v>
       </c>
     </row>
-    <row r="158" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:12">
       <c r="A158" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B158" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C158">
         <v>30</v>
@@ -5516,12 +5516,12 @@
         <v>26610</v>
       </c>
     </row>
-    <row r="159" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:12">
       <c r="A159" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B159" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C159">
         <v>33</v>
@@ -5554,12 +5554,12 @@
         <v>28560</v>
       </c>
     </row>
-    <row r="160" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:12">
       <c r="A160" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B160" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C160">
         <v>39</v>
@@ -5592,12 +5592,12 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="161" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:12">
       <c r="A161" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B161" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C161">
         <v>45</v>
@@ -5630,12 +5630,12 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="162" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="162" spans="1:12">
       <c r="A162" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B162" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C162">
         <v>32</v>
@@ -5668,12 +5668,12 @@
         <v>27910</v>
       </c>
     </row>
-    <row r="163" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="163" spans="1:12">
       <c r="A163" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B163" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C163">
         <v>35</v>
@@ -5706,12 +5706,12 @@
         <v>29880</v>
       </c>
     </row>
-    <row r="164" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="164" spans="1:12">
       <c r="A164" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B164" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C164">
         <v>41</v>
@@ -5744,12 +5744,12 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="165" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:12">
       <c r="A165" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B165" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C165">
         <v>38</v>
@@ -5782,12 +5782,12 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="166" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:12">
       <c r="A166" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B166" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C166">
         <v>44</v>
@@ -5820,12 +5820,12 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="167" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:12">
       <c r="A167" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B167" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C167">
         <v>34</v>
@@ -5858,12 +5858,12 @@
         <v>29260</v>
       </c>
     </row>
-    <row r="168" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="168" spans="1:12">
       <c r="A168" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B168" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C168">
         <v>37</v>
@@ -5896,12 +5896,12 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="169" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="169" spans="1:12">
       <c r="A169" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B169" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C169">
         <v>43</v>
@@ -5934,12 +5934,12 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="170" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="170" spans="1:12">
       <c r="A170" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B170" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C170">
         <v>40</v>
@@ -5972,12 +5972,12 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="171" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="171" spans="1:12">
       <c r="A171" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B171" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C171">
         <v>46</v>
@@ -6010,12 +6010,12 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="172" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="172" spans="1:12">
       <c r="A172" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B172" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C172">
         <v>43</v>
@@ -6048,12 +6048,12 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="173" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="173" spans="1:12">
       <c r="A173" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B173" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C173">
         <v>36</v>
@@ -6086,12 +6086,12 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="174" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="174" spans="1:12">
       <c r="A174" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B174" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C174">
         <v>39</v>
@@ -6124,12 +6124,12 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="175" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="175" spans="1:12">
       <c r="A175" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B175" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C175">
         <v>45</v>
@@ -6162,12 +6162,12 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="176" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="176" spans="1:12">
       <c r="A176" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B176" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C176">
         <v>42</v>
@@ -6200,12 +6200,12 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="177" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="177" spans="1:12">
       <c r="A177" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B177" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C177">
         <v>45</v>
@@ -6247,39 +6247,39 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D46"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.45"/>
   <cols>
-    <col min="1" max="1" width="15.26953125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="21.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16.453125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="19.90625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4">
       <c r="A1" s="2" t="s">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
       <c r="D1" s="2"/>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:4">
       <c r="A2" t="s">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="B2" t="s">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="C2" t="s">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="D2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
       <c r="A3" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B3">
         <v>46</v>
@@ -6291,9 +6291,9 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:4">
       <c r="A4" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B4">
         <v>45</v>
@@ -6305,9 +6305,9 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:4">
       <c r="A5" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B5">
         <v>44</v>
@@ -6319,9 +6319,9 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:4">
       <c r="A6" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B6">
         <v>43</v>
@@ -6333,9 +6333,9 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:4">
       <c r="A7" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B7">
         <v>42</v>
@@ -6347,9 +6347,9 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:4">
       <c r="A8" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B8">
         <v>41</v>
@@ -6361,9 +6361,9 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:4">
       <c r="A9" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B9">
         <v>40</v>
@@ -6375,9 +6375,9 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:4">
       <c r="A10" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B10">
         <v>39</v>
@@ -6389,9 +6389,9 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:4">
       <c r="A11" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B11">
         <v>38</v>
@@ -6403,9 +6403,9 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:4">
       <c r="A12" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B12">
         <v>37</v>
@@ -6417,9 +6417,9 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:4">
       <c r="A13" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B13">
         <v>36</v>
@@ -6431,9 +6431,9 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:4">
       <c r="A14" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B14">
         <v>35</v>
@@ -6445,9 +6445,9 @@
         <v>29880</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:4">
       <c r="A15" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B15">
         <v>34</v>
@@ -6459,9 +6459,9 @@
         <v>29260</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:4">
       <c r="A16" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B16">
         <v>33</v>
@@ -6473,9 +6473,9 @@
         <v>28560</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:4">
       <c r="A17" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B17">
         <v>32</v>
@@ -6487,9 +6487,9 @@
         <v>27910</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:4">
       <c r="A18" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B18">
         <v>31</v>
@@ -6501,9 +6501,9 @@
         <v>27260</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:4">
       <c r="A19" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B19">
         <v>30</v>
@@ -6515,9 +6515,9 @@
         <v>26610</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:4">
       <c r="A20" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B20">
         <v>29</v>
@@ -6529,9 +6529,9 @@
         <v>25960</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:4">
       <c r="A21" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B21">
         <v>28</v>
@@ -6543,9 +6543,9 @@
         <v>25310</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:4">
       <c r="A22" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B22">
         <v>27</v>
@@ -6557,9 +6557,9 @@
         <v>24660</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:4">
       <c r="A23" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B23">
         <v>26</v>
@@ -6571,9 +6571,9 @@
         <v>24010</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:4">
       <c r="A24" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B24">
         <v>25</v>
@@ -6585,9 +6585,9 @@
         <v>23360</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:4">
       <c r="A25" t="s">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="B25">
         <v>31</v>
@@ -6599,9 +6599,9 @@
         <v>22505</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:4">
       <c r="A26" t="s">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="B26">
         <v>30</v>
@@ -6613,9 +6613,9 @@
         <v>22505</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:4">
       <c r="A27" t="s">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="B27">
         <v>29</v>
@@ -6627,9 +6627,9 @@
         <v>22505</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:4">
       <c r="A28" t="s">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="B28">
         <v>28</v>
@@ -6641,9 +6641,9 @@
         <v>22505</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:4">
       <c r="A29" t="s">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="B29">
         <v>27</v>
@@ -6655,9 +6655,9 @@
         <v>22505</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:4">
       <c r="A30" t="s">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="B30">
         <v>26</v>
@@ -6669,9 +6669,9 @@
         <v>22505</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:4">
       <c r="A31" t="s">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="B31">
         <v>25</v>
@@ -6683,9 +6683,9 @@
         <v>22505</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:4">
       <c r="A32" t="s">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="B32">
         <v>24</v>
@@ -6697,9 +6697,9 @@
         <v>22505</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:4">
       <c r="A33" t="s">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="B33">
         <v>23</v>
@@ -6711,9 +6711,9 @@
         <v>22505</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:4">
       <c r="A34" t="s">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="B34">
         <v>22</v>
@@ -6725,9 +6725,9 @@
         <v>21630</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:4">
       <c r="A35" t="s">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="B35">
         <v>21</v>
@@ -6739,9 +6739,9 @@
         <v>20690</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:4">
       <c r="A36" t="s">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="B36">
         <v>19</v>
@@ -6753,9 +6753,9 @@
         <v>19165</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:4">
       <c r="A37" t="s">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="B37">
         <v>18</v>
@@ -6767,9 +6767,9 @@
         <v>18440</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:4">
       <c r="A38" t="s">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="B38">
         <v>16</v>
@@ -6781,9 +6781,9 @@
         <v>17785</v>
       </c>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:4">
       <c r="A39" t="s">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="B39">
         <v>14</v>
@@ -6795,9 +6795,9 @@
         <v>16115</v>
       </c>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:4">
       <c r="A40" t="s">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="B40">
         <v>24</v>
@@ -6809,9 +6809,9 @@
         <v>19725</v>
       </c>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:4">
       <c r="A41" t="s">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="B41">
         <v>22</v>
@@ -6823,9 +6823,9 @@
         <v>19725</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:4">
       <c r="A42" t="s">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="B42">
         <v>21</v>
@@ -6837,9 +6837,9 @@
         <v>19725</v>
       </c>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:4">
       <c r="A43" t="s">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="B43">
         <v>19</v>
@@ -6851,9 +6851,9 @@
         <v>19725</v>
       </c>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:4">
       <c r="A44" t="s">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="B44">
         <v>18</v>
@@ -6865,9 +6865,9 @@
         <v>19725</v>
       </c>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:4">
       <c r="A45" t="s">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="B45">
         <v>16</v>
@@ -6879,9 +6879,9 @@
         <v>17750</v>
       </c>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:4">
       <c r="A46" t="s">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="B46">
         <v>14</v>

</xml_diff>

<commit_message>
change so heads/rooms starts at 1 and added single units for both manufacturers
</commit_message>
<xml_diff>
--- a/backend/assets/data/fujitsu_capacities_calculated.xlsx
+++ b/backend/assets/data/fujitsu_capacities_calculated.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29609"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AlexWest\OneDrive - Paradigm Energy Services\data_operations\ashp_calculator\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://pardigmpartners-my.sharepoint.com/personal/alex_paradigm-esco_com/Documents/data_operations/ashp_calculator/backend/assets/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D420F103-AC1D-4B35-A441-D57FBF080E0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="26" documentId="13_ncr:1_{D420F103-AC1D-4B35-A441-D57FBF080E0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7573420A-3779-4C44-8361-9FBDA80001B9}"/>
   <bookViews>
-    <workbookView xWindow="4940" yWindow="1440" windowWidth="30890" windowHeight="17110" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="6110" yWindow="820" windowWidth="30890" windowHeight="17460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="indoor_combinations" sheetId="2" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="413" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="425" uniqueCount="27">
   <si>
     <t>Model</t>
   </si>
@@ -101,12 +101,30 @@
   <si>
     <t>Capacity at 70F (Btu/h)</t>
   </si>
+  <si>
+    <t>AOUH12KUAS1</t>
+  </si>
+  <si>
+    <t>AOUH18KUAS1</t>
+  </si>
+  <si>
+    <t>AOUH24KUAS1</t>
+  </si>
+  <si>
+    <t>AOUH30KUAS1</t>
+  </si>
+  <si>
+    <t>AOUH36KUAS1</t>
+  </si>
+  <si>
+    <t>AOUH48KUAS1</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -141,11 +159,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -427,20 +451,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2E4304B4-14C5-40DF-85A6-AED3FDED911B}">
-  <dimension ref="A1:N177"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <dimension ref="A1:N183"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="14.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.26953125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="14" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="5.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="5.7109375" customWidth="1"/>
-    <col min="8" max="9" width="17.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="11" width="17.42578125" customWidth="1"/>
-    <col min="12" max="12" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="6.26953125" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="5.7265625" customWidth="1"/>
+    <col min="8" max="9" width="17.453125" bestFit="1" customWidth="1"/>
+    <col min="10" max="11" width="17.453125" customWidth="1"/>
+    <col min="12" max="12" width="12.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -478,7 +502,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:14">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>12</v>
       </c>
@@ -504,7 +528,7 @@
         <v>16335</v>
       </c>
     </row>
-    <row r="3" spans="1:14">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>12</v>
       </c>
@@ -530,7 +554,7 @@
         <v>17750</v>
       </c>
     </row>
-    <row r="4" spans="1:14">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>12</v>
       </c>
@@ -556,7 +580,7 @@
         <v>19725</v>
       </c>
     </row>
-    <row r="5" spans="1:14">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>12</v>
       </c>
@@ -582,7 +606,7 @@
         <v>19725</v>
       </c>
     </row>
-    <row r="6" spans="1:14">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>12</v>
       </c>
@@ -608,7 +632,7 @@
         <v>19725</v>
       </c>
     </row>
-    <row r="7" spans="1:14">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>12</v>
       </c>
@@ -634,7 +658,7 @@
         <v>19725</v>
       </c>
     </row>
-    <row r="8" spans="1:14">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>12</v>
       </c>
@@ -660,7 +684,7 @@
         <v>19725</v>
       </c>
     </row>
-    <row r="9" spans="1:14">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>12</v>
       </c>
@@ -686,7 +710,7 @@
         <v>19725</v>
       </c>
     </row>
-    <row r="10" spans="1:14">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>12</v>
       </c>
@@ -712,7 +736,7 @@
         <v>16335</v>
       </c>
     </row>
-    <row r="11" spans="1:14">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>12</v>
       </c>
@@ -738,7 +762,7 @@
         <v>17750</v>
       </c>
     </row>
-    <row r="12" spans="1:14">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>12</v>
       </c>
@@ -764,7 +788,7 @@
         <v>19725</v>
       </c>
     </row>
-    <row r="13" spans="1:14">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>12</v>
       </c>
@@ -790,7 +814,7 @@
         <v>19725</v>
       </c>
     </row>
-    <row r="14" spans="1:14">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>12</v>
       </c>
@@ -816,7 +840,7 @@
         <v>19725</v>
       </c>
     </row>
-    <row r="15" spans="1:14">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>12</v>
       </c>
@@ -842,7 +866,7 @@
         <v>19725</v>
       </c>
     </row>
-    <row r="16" spans="1:14">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>15</v>
       </c>
@@ -872,7 +896,7 @@
       <c r="M16" s="1"/>
       <c r="N16" s="1"/>
     </row>
-    <row r="17" spans="1:14">
+    <row r="17" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>15</v>
       </c>
@@ -902,7 +926,7 @@
       <c r="M17" s="1"/>
       <c r="N17" s="1"/>
     </row>
-    <row r="18" spans="1:14">
+    <row r="18" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>15</v>
       </c>
@@ -932,7 +956,7 @@
       <c r="M18" s="1"/>
       <c r="N18" s="1"/>
     </row>
-    <row r="19" spans="1:14">
+    <row r="19" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>15</v>
       </c>
@@ -962,7 +986,7 @@
       <c r="M19" s="1"/>
       <c r="N19" s="1"/>
     </row>
-    <row r="20" spans="1:14">
+    <row r="20" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>15</v>
       </c>
@@ -992,7 +1016,7 @@
       <c r="M20" s="1"/>
       <c r="N20" s="1"/>
     </row>
-    <row r="21" spans="1:14">
+    <row r="21" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>15</v>
       </c>
@@ -1022,7 +1046,7 @@
       <c r="M21" s="1"/>
       <c r="N21" s="1"/>
     </row>
-    <row r="22" spans="1:14">
+    <row r="22" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>15</v>
       </c>
@@ -1052,7 +1076,7 @@
       <c r="M22" s="1"/>
       <c r="N22" s="1"/>
     </row>
-    <row r="23" spans="1:14">
+    <row r="23" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>15</v>
       </c>
@@ -1082,7 +1106,7 @@
       <c r="M23" s="1"/>
       <c r="N23" s="1"/>
     </row>
-    <row r="24" spans="1:14">
+    <row r="24" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>15</v>
       </c>
@@ -1112,7 +1136,7 @@
       <c r="M24" s="1"/>
       <c r="N24" s="1"/>
     </row>
-    <row r="25" spans="1:14">
+    <row r="25" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>15</v>
       </c>
@@ -1142,7 +1166,7 @@
       <c r="M25" s="1"/>
       <c r="N25" s="1"/>
     </row>
-    <row r="26" spans="1:14">
+    <row r="26" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>15</v>
       </c>
@@ -1172,7 +1196,7 @@
       <c r="M26" s="1"/>
       <c r="N26" s="1"/>
     </row>
-    <row r="27" spans="1:14">
+    <row r="27" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>15</v>
       </c>
@@ -1202,7 +1226,7 @@
       <c r="M27" s="1"/>
       <c r="N27" s="1"/>
     </row>
-    <row r="28" spans="1:14">
+    <row r="28" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>15</v>
       </c>
@@ -1232,7 +1256,7 @@
       <c r="M28" s="1"/>
       <c r="N28" s="1"/>
     </row>
-    <row r="29" spans="1:14">
+    <row r="29" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>15</v>
       </c>
@@ -1267,7 +1291,7 @@
       <c r="M29" s="1"/>
       <c r="N29" s="1"/>
     </row>
-    <row r="30" spans="1:14">
+    <row r="30" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>15</v>
       </c>
@@ -1302,7 +1326,7 @@
       <c r="M30" s="1"/>
       <c r="N30" s="1"/>
     </row>
-    <row r="31" spans="1:14">
+    <row r="31" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>15</v>
       </c>
@@ -1337,7 +1361,7 @@
       <c r="M31" s="1"/>
       <c r="N31" s="1"/>
     </row>
-    <row r="32" spans="1:14">
+    <row r="32" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>15</v>
       </c>
@@ -1372,7 +1396,7 @@
       <c r="M32" s="1"/>
       <c r="N32" s="1"/>
     </row>
-    <row r="33" spans="1:14">
+    <row r="33" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>15</v>
       </c>
@@ -1407,7 +1431,7 @@
       <c r="M33" s="1"/>
       <c r="N33" s="1"/>
     </row>
-    <row r="34" spans="1:14">
+    <row r="34" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>15</v>
       </c>
@@ -1442,7 +1466,7 @@
       <c r="M34" s="1"/>
       <c r="N34" s="1"/>
     </row>
-    <row r="35" spans="1:14">
+    <row r="35" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>15</v>
       </c>
@@ -1477,7 +1501,7 @@
       <c r="M35" s="1"/>
       <c r="N35" s="1"/>
     </row>
-    <row r="36" spans="1:14">
+    <row r="36" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>15</v>
       </c>
@@ -1512,7 +1536,7 @@
       <c r="M36" s="1"/>
       <c r="N36" s="1"/>
     </row>
-    <row r="37" spans="1:14">
+    <row r="37" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>15</v>
       </c>
@@ -1547,7 +1571,7 @@
       <c r="M37" s="1"/>
       <c r="N37" s="1"/>
     </row>
-    <row r="38" spans="1:14">
+    <row r="38" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>15</v>
       </c>
@@ -1582,7 +1606,7 @@
       <c r="M38" s="1"/>
       <c r="N38" s="1"/>
     </row>
-    <row r="39" spans="1:14">
+    <row r="39" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>15</v>
       </c>
@@ -1610,7 +1634,7 @@
         <v>16115</v>
       </c>
     </row>
-    <row r="40" spans="1:14">
+    <row r="40" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>15</v>
       </c>
@@ -1638,7 +1662,7 @@
         <v>17785</v>
       </c>
     </row>
-    <row r="41" spans="1:14">
+    <row r="41" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>15</v>
       </c>
@@ -1666,7 +1690,7 @@
         <v>19165</v>
       </c>
     </row>
-    <row r="42" spans="1:14">
+    <row r="42" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>15</v>
       </c>
@@ -1694,7 +1718,7 @@
         <v>22505</v>
       </c>
     </row>
-    <row r="43" spans="1:14">
+    <row r="43" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>15</v>
       </c>
@@ -1722,7 +1746,7 @@
         <v>18440</v>
       </c>
     </row>
-    <row r="44" spans="1:14">
+    <row r="44" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>15</v>
       </c>
@@ -1750,7 +1774,7 @@
         <v>20690</v>
       </c>
     </row>
-    <row r="45" spans="1:14">
+    <row r="45" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>15</v>
       </c>
@@ -1778,7 +1802,7 @@
         <v>22505</v>
       </c>
     </row>
-    <row r="46" spans="1:14">
+    <row r="46" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>15</v>
       </c>
@@ -1806,7 +1830,7 @@
         <v>22505</v>
       </c>
     </row>
-    <row r="47" spans="1:14">
+    <row r="47" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>15</v>
       </c>
@@ -1834,7 +1858,7 @@
         <v>22505</v>
       </c>
     </row>
-    <row r="48" spans="1:14">
+    <row r="48" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>15</v>
       </c>
@@ -1868,7 +1892,7 @@
         <v>20690</v>
       </c>
     </row>
-    <row r="49" spans="1:12">
+    <row r="49" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>15</v>
       </c>
@@ -1902,7 +1926,7 @@
         <v>22505</v>
       </c>
     </row>
-    <row r="50" spans="1:12">
+    <row r="50" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>15</v>
       </c>
@@ -1936,7 +1960,7 @@
         <v>22505</v>
       </c>
     </row>
-    <row r="51" spans="1:12">
+    <row r="51" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>15</v>
       </c>
@@ -1970,7 +1994,7 @@
         <v>22505</v>
       </c>
     </row>
-    <row r="52" spans="1:12">
+    <row r="52" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>15</v>
       </c>
@@ -2004,7 +2028,7 @@
         <v>22505</v>
       </c>
     </row>
-    <row r="53" spans="1:12">
+    <row r="53" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>15</v>
       </c>
@@ -2038,7 +2062,7 @@
         <v>22505</v>
       </c>
     </row>
-    <row r="54" spans="1:12">
+    <row r="54" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>15</v>
       </c>
@@ -2072,7 +2096,7 @@
         <v>22505</v>
       </c>
     </row>
-    <row r="55" spans="1:12">
+    <row r="55" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>15</v>
       </c>
@@ -2106,7 +2130,7 @@
         <v>22505</v>
       </c>
     </row>
-    <row r="56" spans="1:12">
+    <row r="56" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
         <v>16</v>
       </c>
@@ -2132,7 +2156,7 @@
         <v>27260</v>
       </c>
     </row>
-    <row r="57" spans="1:12">
+    <row r="57" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
         <v>16</v>
       </c>
@@ -2158,7 +2182,7 @@
         <v>28560</v>
       </c>
     </row>
-    <row r="58" spans="1:12">
+    <row r="58" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
         <v>16</v>
       </c>
@@ -2184,7 +2208,7 @@
         <v>26610</v>
       </c>
     </row>
-    <row r="59" spans="1:12">
+    <row r="59" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
         <v>16</v>
       </c>
@@ -2210,7 +2234,7 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="60" spans="1:12">
+    <row r="60" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
         <v>16</v>
       </c>
@@ -2236,7 +2260,7 @@
         <v>28560</v>
       </c>
     </row>
-    <row r="61" spans="1:12">
+    <row r="61" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
         <v>16</v>
       </c>
@@ -2262,7 +2286,7 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="62" spans="1:12">
+    <row r="62" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
         <v>16</v>
       </c>
@@ -2288,7 +2312,7 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="63" spans="1:12">
+    <row r="63" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
         <v>16</v>
       </c>
@@ -2314,7 +2338,7 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="64" spans="1:12">
+    <row r="64" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
         <v>16</v>
       </c>
@@ -2346,7 +2370,7 @@
         <v>24010</v>
       </c>
     </row>
-    <row r="65" spans="1:12">
+    <row r="65" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
         <v>16</v>
       </c>
@@ -2378,7 +2402,7 @@
         <v>25960</v>
       </c>
     </row>
-    <row r="66" spans="1:12">
+    <row r="66" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
         <v>16</v>
       </c>
@@ -2410,7 +2434,7 @@
         <v>27910</v>
       </c>
     </row>
-    <row r="67" spans="1:12">
+    <row r="67" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
         <v>16</v>
       </c>
@@ -2442,7 +2466,7 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="68" spans="1:12">
+    <row r="68" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
         <v>16</v>
       </c>
@@ -2474,7 +2498,7 @@
         <v>23360</v>
       </c>
     </row>
-    <row r="69" spans="1:12">
+    <row r="69" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
         <v>16</v>
       </c>
@@ -2506,7 +2530,7 @@
         <v>25310</v>
       </c>
     </row>
-    <row r="70" spans="1:12">
+    <row r="70" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
         <v>16</v>
       </c>
@@ -2538,7 +2562,7 @@
         <v>27260</v>
       </c>
     </row>
-    <row r="71" spans="1:12">
+    <row r="71" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
         <v>16</v>
       </c>
@@ -2570,7 +2594,7 @@
         <v>29260</v>
       </c>
     </row>
-    <row r="72" spans="1:12">
+    <row r="72" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
         <v>16</v>
       </c>
@@ -2602,7 +2626,7 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="73" spans="1:12">
+    <row r="73" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
         <v>16</v>
       </c>
@@ -2634,7 +2658,7 @@
         <v>27260</v>
       </c>
     </row>
-    <row r="74" spans="1:12">
+    <row r="74" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
         <v>16</v>
       </c>
@@ -2666,7 +2690,7 @@
         <v>29260</v>
       </c>
     </row>
-    <row r="75" spans="1:12">
+    <row r="75" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
         <v>16</v>
       </c>
@@ -2698,7 +2722,7 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="76" spans="1:12">
+    <row r="76" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
         <v>16</v>
       </c>
@@ -2730,7 +2754,7 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="77" spans="1:12">
+    <row r="77" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
         <v>16</v>
       </c>
@@ -2762,7 +2786,7 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="78" spans="1:12">
+    <row r="78" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
         <v>16</v>
       </c>
@@ -2794,7 +2818,7 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="79" spans="1:12">
+    <row r="79" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
         <v>16</v>
       </c>
@@ -2826,7 +2850,7 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="80" spans="1:12">
+    <row r="80" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
         <v>16</v>
       </c>
@@ -2858,7 +2882,7 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="81" spans="1:12">
+    <row r="81" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
         <v>16</v>
       </c>
@@ -2890,7 +2914,7 @@
         <v>24660</v>
       </c>
     </row>
-    <row r="82" spans="1:12">
+    <row r="82" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
         <v>16</v>
       </c>
@@ -2922,7 +2946,7 @@
         <v>26610</v>
       </c>
     </row>
-    <row r="83" spans="1:12">
+    <row r="83" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A83" t="s">
         <v>16</v>
       </c>
@@ -2954,7 +2978,7 @@
         <v>28560</v>
       </c>
     </row>
-    <row r="84" spans="1:12">
+    <row r="84" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A84" t="s">
         <v>16</v>
       </c>
@@ -2986,7 +3010,7 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="85" spans="1:12">
+    <row r="85" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A85" t="s">
         <v>16</v>
       </c>
@@ -3018,7 +3042,7 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="86" spans="1:12">
+    <row r="86" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A86" t="s">
         <v>16</v>
       </c>
@@ -3050,7 +3074,7 @@
         <v>28560</v>
       </c>
     </row>
-    <row r="87" spans="1:12">
+    <row r="87" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A87" t="s">
         <v>16</v>
       </c>
@@ -3082,7 +3106,7 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="88" spans="1:12">
+    <row r="88" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A88" t="s">
         <v>16</v>
       </c>
@@ -3114,7 +3138,7 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="89" spans="1:12">
+    <row r="89" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A89" t="s">
         <v>16</v>
       </c>
@@ -3146,7 +3170,7 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="90" spans="1:12">
+    <row r="90" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A90" t="s">
         <v>16</v>
       </c>
@@ -3178,7 +3202,7 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="91" spans="1:12">
+    <row r="91" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A91" t="s">
         <v>16</v>
       </c>
@@ -3210,7 +3234,7 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="92" spans="1:12">
+    <row r="92" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A92" t="s">
         <v>16</v>
       </c>
@@ -3242,7 +3266,7 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="93" spans="1:12">
+    <row r="93" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A93" t="s">
         <v>16</v>
       </c>
@@ -3274,7 +3298,7 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="94" spans="1:12">
+    <row r="94" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A94" t="s">
         <v>16</v>
       </c>
@@ -3306,7 +3330,7 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="95" spans="1:12">
+    <row r="95" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A95" t="s">
         <v>16</v>
       </c>
@@ -3338,7 +3362,7 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="96" spans="1:12">
+    <row r="96" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A96" t="s">
         <v>16</v>
       </c>
@@ -3370,7 +3394,7 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="97" spans="1:12">
+    <row r="97" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A97" t="s">
         <v>16</v>
       </c>
@@ -3402,7 +3426,7 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="98" spans="1:12">
+    <row r="98" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A98" t="s">
         <v>16</v>
       </c>
@@ -3434,7 +3458,7 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="99" spans="1:12">
+    <row r="99" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A99" t="s">
         <v>16</v>
       </c>
@@ -3472,7 +3496,7 @@
         <v>25310</v>
       </c>
     </row>
-    <row r="100" spans="1:12">
+    <row r="100" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A100" t="s">
         <v>16</v>
       </c>
@@ -3510,7 +3534,7 @@
         <v>26610</v>
       </c>
     </row>
-    <row r="101" spans="1:12">
+    <row r="101" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A101" t="s">
         <v>16</v>
       </c>
@@ -3548,7 +3572,7 @@
         <v>28560</v>
       </c>
     </row>
-    <row r="102" spans="1:12">
+    <row r="102" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A102" t="s">
         <v>16</v>
       </c>
@@ -3586,7 +3610,7 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="103" spans="1:12">
+    <row r="103" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A103" t="s">
         <v>16</v>
       </c>
@@ -3624,7 +3648,7 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="104" spans="1:12">
+    <row r="104" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A104" t="s">
         <v>16</v>
       </c>
@@ -3662,7 +3686,7 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="105" spans="1:12">
+    <row r="105" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A105" t="s">
         <v>16</v>
       </c>
@@ -3700,7 +3724,7 @@
         <v>27910</v>
       </c>
     </row>
-    <row r="106" spans="1:12">
+    <row r="106" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A106" t="s">
         <v>16</v>
       </c>
@@ -3738,7 +3762,7 @@
         <v>29880</v>
       </c>
     </row>
-    <row r="107" spans="1:12">
+    <row r="107" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A107" t="s">
         <v>16</v>
       </c>
@@ -3776,7 +3800,7 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="108" spans="1:12">
+    <row r="108" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A108" t="s">
         <v>16</v>
       </c>
@@ -3814,7 +3838,7 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="109" spans="1:12">
+    <row r="109" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A109" t="s">
         <v>16</v>
       </c>
@@ -3852,7 +3876,7 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="110" spans="1:12">
+    <row r="110" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A110" t="s">
         <v>16</v>
       </c>
@@ -3890,7 +3914,7 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="111" spans="1:12">
+    <row r="111" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A111" t="s">
         <v>16</v>
       </c>
@@ -3928,7 +3952,7 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="112" spans="1:12">
+    <row r="112" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A112" t="s">
         <v>16</v>
       </c>
@@ -3966,7 +3990,7 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="113" spans="1:12">
+    <row r="113" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A113" t="s">
         <v>16</v>
       </c>
@@ -4004,7 +4028,7 @@
         <v>29260</v>
       </c>
     </row>
-    <row r="114" spans="1:12">
+    <row r="114" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A114" t="s">
         <v>16</v>
       </c>
@@ -4042,7 +4066,7 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="115" spans="1:12">
+    <row r="115" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A115" t="s">
         <v>16</v>
       </c>
@@ -4080,7 +4104,7 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="116" spans="1:12">
+    <row r="116" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A116" t="s">
         <v>16</v>
       </c>
@@ -4118,7 +4142,7 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="117" spans="1:12">
+    <row r="117" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A117" t="s">
         <v>16</v>
       </c>
@@ -4156,7 +4180,7 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="118" spans="1:12">
+    <row r="118" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A118" t="s">
         <v>16</v>
       </c>
@@ -4194,7 +4218,7 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="119" spans="1:12">
+    <row r="119" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A119" t="s">
         <v>16</v>
       </c>
@@ -4232,7 +4256,7 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="120" spans="1:12">
+    <row r="120" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A120" t="s">
         <v>16</v>
       </c>
@@ -4270,7 +4294,7 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="121" spans="1:12">
+    <row r="121" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A121" t="s">
         <v>16</v>
       </c>
@@ -4308,7 +4332,7 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="122" spans="1:12">
+    <row r="122" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A122" t="s">
         <v>16</v>
       </c>
@@ -4346,7 +4370,7 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="123" spans="1:12">
+    <row r="123" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A123" t="s">
         <v>16</v>
       </c>
@@ -4384,7 +4408,7 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="124" spans="1:12">
+    <row r="124" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A124" t="s">
         <v>16</v>
       </c>
@@ -4422,7 +4446,7 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="125" spans="1:12">
+    <row r="125" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A125" t="s">
         <v>16</v>
       </c>
@@ -4460,7 +4484,7 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="126" spans="1:12">
+    <row r="126" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A126" t="s">
         <v>16</v>
       </c>
@@ -4498,7 +4522,7 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="127" spans="1:12">
+    <row r="127" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A127" t="s">
         <v>16</v>
       </c>
@@ -4536,7 +4560,7 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="128" spans="1:12">
+    <row r="128" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A128" t="s">
         <v>16</v>
       </c>
@@ -4574,7 +4598,7 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="129" spans="1:12">
+    <row r="129" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A129" t="s">
         <v>16</v>
       </c>
@@ -4612,7 +4636,7 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="130" spans="1:12">
+    <row r="130" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A130" t="s">
         <v>16</v>
       </c>
@@ -4638,7 +4662,7 @@
         <v>27260</v>
       </c>
     </row>
-    <row r="131" spans="1:12">
+    <row r="131" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A131" t="s">
         <v>16</v>
       </c>
@@ -4664,7 +4688,7 @@
         <v>28560</v>
       </c>
     </row>
-    <row r="132" spans="1:12">
+    <row r="132" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A132" t="s">
         <v>16</v>
       </c>
@@ -4690,7 +4714,7 @@
         <v>26610</v>
       </c>
     </row>
-    <row r="133" spans="1:12">
+    <row r="133" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A133" t="s">
         <v>16</v>
       </c>
@@ -4716,7 +4740,7 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="134" spans="1:12">
+    <row r="134" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A134" t="s">
         <v>16</v>
       </c>
@@ -4742,7 +4766,7 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="135" spans="1:12">
+    <row r="135" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A135" t="s">
         <v>16</v>
       </c>
@@ -4768,7 +4792,7 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="136" spans="1:12">
+    <row r="136" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A136" t="s">
         <v>16</v>
       </c>
@@ -4800,7 +4824,7 @@
         <v>24010</v>
       </c>
     </row>
-    <row r="137" spans="1:12">
+    <row r="137" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A137" t="s">
         <v>16</v>
       </c>
@@ -4832,7 +4856,7 @@
         <v>27910</v>
       </c>
     </row>
-    <row r="138" spans="1:12">
+    <row r="138" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A138" t="s">
         <v>16</v>
       </c>
@@ -4864,7 +4888,7 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="139" spans="1:12">
+    <row r="139" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A139" t="s">
         <v>16</v>
       </c>
@@ -4896,7 +4920,7 @@
         <v>23360</v>
       </c>
     </row>
-    <row r="140" spans="1:12">
+    <row r="140" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A140" t="s">
         <v>16</v>
       </c>
@@ -4928,7 +4952,7 @@
         <v>25310</v>
       </c>
     </row>
-    <row r="141" spans="1:12">
+    <row r="141" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A141" t="s">
         <v>16</v>
       </c>
@@ -4960,7 +4984,7 @@
         <v>29260</v>
       </c>
     </row>
-    <row r="142" spans="1:12">
+    <row r="142" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A142" t="s">
         <v>16</v>
       </c>
@@ -4992,7 +5016,7 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="143" spans="1:12">
+    <row r="143" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A143" t="s">
         <v>16</v>
       </c>
@@ -5024,7 +5048,7 @@
         <v>27260</v>
       </c>
     </row>
-    <row r="144" spans="1:12">
+    <row r="144" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A144" t="s">
         <v>16</v>
       </c>
@@ -5056,7 +5080,7 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="145" spans="1:12">
+    <row r="145" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A145" t="s">
         <v>16</v>
       </c>
@@ -5088,7 +5112,7 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="146" spans="1:12">
+    <row r="146" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A146" t="s">
         <v>16</v>
       </c>
@@ -5120,7 +5144,7 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="147" spans="1:12">
+    <row r="147" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A147" t="s">
         <v>16</v>
       </c>
@@ -5152,7 +5176,7 @@
         <v>24660</v>
       </c>
     </row>
-    <row r="148" spans="1:12">
+    <row r="148" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A148" t="s">
         <v>16</v>
       </c>
@@ -5184,7 +5208,7 @@
         <v>26610</v>
       </c>
     </row>
-    <row r="149" spans="1:12">
+    <row r="149" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A149" t="s">
         <v>16</v>
       </c>
@@ -5216,7 +5240,7 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="150" spans="1:12">
+    <row r="150" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A150" t="s">
         <v>16</v>
       </c>
@@ -5248,7 +5272,7 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="151" spans="1:12">
+    <row r="151" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A151" t="s">
         <v>16</v>
       </c>
@@ -5280,7 +5304,7 @@
         <v>28560</v>
       </c>
     </row>
-    <row r="152" spans="1:12">
+    <row r="152" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A152" t="s">
         <v>16</v>
       </c>
@@ -5312,7 +5336,7 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="153" spans="1:12">
+    <row r="153" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A153" t="s">
         <v>16</v>
       </c>
@@ -5344,7 +5368,7 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="154" spans="1:12">
+    <row r="154" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A154" t="s">
         <v>16</v>
       </c>
@@ -5376,7 +5400,7 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="155" spans="1:12">
+    <row r="155" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A155" t="s">
         <v>16</v>
       </c>
@@ -5408,7 +5432,7 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="156" spans="1:12">
+    <row r="156" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A156" t="s">
         <v>16</v>
       </c>
@@ -5440,7 +5464,7 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="157" spans="1:12">
+    <row r="157" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A157" t="s">
         <v>16</v>
       </c>
@@ -5478,7 +5502,7 @@
         <v>25310</v>
       </c>
     </row>
-    <row r="158" spans="1:12">
+    <row r="158" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A158" t="s">
         <v>16</v>
       </c>
@@ -5516,7 +5540,7 @@
         <v>26610</v>
       </c>
     </row>
-    <row r="159" spans="1:12">
+    <row r="159" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A159" t="s">
         <v>16</v>
       </c>
@@ -5554,7 +5578,7 @@
         <v>28560</v>
       </c>
     </row>
-    <row r="160" spans="1:12">
+    <row r="160" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A160" t="s">
         <v>16</v>
       </c>
@@ -5592,7 +5616,7 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="161" spans="1:12">
+    <row r="161" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A161" t="s">
         <v>16</v>
       </c>
@@ -5630,7 +5654,7 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="162" spans="1:12">
+    <row r="162" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A162" t="s">
         <v>16</v>
       </c>
@@ -5668,7 +5692,7 @@
         <v>27910</v>
       </c>
     </row>
-    <row r="163" spans="1:12">
+    <row r="163" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A163" t="s">
         <v>16</v>
       </c>
@@ -5706,7 +5730,7 @@
         <v>29880</v>
       </c>
     </row>
-    <row r="164" spans="1:12">
+    <row r="164" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A164" t="s">
         <v>16</v>
       </c>
@@ -5744,7 +5768,7 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="165" spans="1:12">
+    <row r="165" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A165" t="s">
         <v>16</v>
       </c>
@@ -5782,7 +5806,7 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="166" spans="1:12">
+    <row r="166" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A166" t="s">
         <v>16</v>
       </c>
@@ -5820,7 +5844,7 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="167" spans="1:12">
+    <row r="167" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A167" t="s">
         <v>16</v>
       </c>
@@ -5858,7 +5882,7 @@
         <v>29260</v>
       </c>
     </row>
-    <row r="168" spans="1:12">
+    <row r="168" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A168" t="s">
         <v>16</v>
       </c>
@@ -5896,7 +5920,7 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="169" spans="1:12">
+    <row r="169" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A169" t="s">
         <v>16</v>
       </c>
@@ -5934,7 +5958,7 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="170" spans="1:12">
+    <row r="170" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A170" t="s">
         <v>16</v>
       </c>
@@ -5972,7 +5996,7 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="171" spans="1:12">
+    <row r="171" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A171" t="s">
         <v>16</v>
       </c>
@@ -6010,7 +6034,7 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="172" spans="1:12">
+    <row r="172" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A172" t="s">
         <v>16</v>
       </c>
@@ -6048,7 +6072,7 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="173" spans="1:12">
+    <row r="173" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A173" t="s">
         <v>16</v>
       </c>
@@ -6086,7 +6110,7 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="174" spans="1:12">
+    <row r="174" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A174" t="s">
         <v>16</v>
       </c>
@@ -6124,7 +6148,7 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="175" spans="1:12">
+    <row r="175" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A175" t="s">
         <v>16</v>
       </c>
@@ -6162,7 +6186,7 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="176" spans="1:12">
+    <row r="176" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A176" t="s">
         <v>16</v>
       </c>
@@ -6200,7 +6224,7 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="177" spans="1:12">
+    <row r="177" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A177" t="s">
         <v>16</v>
       </c>
@@ -6236,6 +6260,156 @@
       </c>
       <c r="L177" s="1">
         <v>30760</v>
+      </c>
+    </row>
+    <row r="178" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A178" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B178" t="s">
+        <v>14</v>
+      </c>
+      <c r="C178" s="3">
+        <v>12</v>
+      </c>
+      <c r="D178" s="3">
+        <v>12</v>
+      </c>
+      <c r="E178" s="4"/>
+      <c r="F178" s="3"/>
+      <c r="G178" s="3"/>
+      <c r="H178" s="4">
+        <v>15310</v>
+      </c>
+      <c r="I178" s="3"/>
+      <c r="J178" s="3"/>
+      <c r="L178" s="4">
+        <v>15310</v>
+      </c>
+    </row>
+    <row r="179" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A179" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B179" t="s">
+        <v>14</v>
+      </c>
+      <c r="C179" s="3">
+        <v>18</v>
+      </c>
+      <c r="D179" s="3">
+        <v>18</v>
+      </c>
+      <c r="E179" s="4"/>
+      <c r="F179" s="3"/>
+      <c r="G179" s="3"/>
+      <c r="H179" s="4">
+        <v>15935</v>
+      </c>
+      <c r="I179" s="3"/>
+      <c r="J179" s="3"/>
+      <c r="L179" s="4">
+        <v>15935</v>
+      </c>
+    </row>
+    <row r="180" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A180" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B180" t="s">
+        <v>14</v>
+      </c>
+      <c r="C180" s="3">
+        <v>24</v>
+      </c>
+      <c r="D180" s="3">
+        <v>24</v>
+      </c>
+      <c r="E180" s="4"/>
+      <c r="F180" s="3"/>
+      <c r="G180" s="3"/>
+      <c r="H180" s="4">
+        <v>23230</v>
+      </c>
+      <c r="I180" s="3"/>
+      <c r="J180" s="3"/>
+      <c r="L180" s="4">
+        <v>23230</v>
+      </c>
+    </row>
+    <row r="181" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A181" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B181" t="s">
+        <v>14</v>
+      </c>
+      <c r="C181" s="3">
+        <v>30</v>
+      </c>
+      <c r="D181" s="3">
+        <v>30</v>
+      </c>
+      <c r="E181" s="4"/>
+      <c r="F181" s="3"/>
+      <c r="G181" s="3"/>
+      <c r="H181" s="4">
+        <v>27295</v>
+      </c>
+      <c r="I181" s="3"/>
+      <c r="J181" s="3"/>
+      <c r="L181" s="4">
+        <v>27295</v>
+      </c>
+    </row>
+    <row r="182" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A182" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B182" t="s">
+        <v>14</v>
+      </c>
+      <c r="C182" s="3">
+        <v>36</v>
+      </c>
+      <c r="D182" s="3">
+        <v>36</v>
+      </c>
+      <c r="E182" s="4"/>
+      <c r="F182" s="3"/>
+      <c r="G182" s="3"/>
+      <c r="H182" s="4">
+        <v>29925</v>
+      </c>
+      <c r="I182" s="3"/>
+      <c r="J182" s="3"/>
+      <c r="L182" s="4">
+        <v>29925</v>
+      </c>
+    </row>
+    <row r="183" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A183" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B183" t="s">
+        <v>14</v>
+      </c>
+      <c r="C183" s="3">
+        <v>48</v>
+      </c>
+      <c r="D183" s="3">
+        <v>48</v>
+      </c>
+      <c r="E183" s="4"/>
+      <c r="F183" s="3"/>
+      <c r="G183" s="3"/>
+      <c r="H183" s="4">
+        <v>39480</v>
+      </c>
+      <c r="I183" s="3"/>
+      <c r="J183" s="3"/>
+      <c r="L183" s="4">
+        <v>39480</v>
       </c>
     </row>
   </sheetData>
@@ -6247,15 +6421,15 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D46"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="15.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="21.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.26953125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.453125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>17</v>
       </c>
@@ -6263,7 +6437,7 @@
       <c r="C1" s="2"/>
       <c r="D1" s="2"/>
     </row>
-    <row r="2" spans="1:4">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -6277,7 +6451,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="3" spans="1:4">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>16</v>
       </c>
@@ -6291,7 +6465,7 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="4" spans="1:4">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>16</v>
       </c>
@@ -6305,7 +6479,7 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="5" spans="1:4">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>16</v>
       </c>
@@ -6319,7 +6493,7 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="6" spans="1:4">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>16</v>
       </c>
@@ -6333,7 +6507,7 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="7" spans="1:4">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>16</v>
       </c>
@@ -6347,7 +6521,7 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="8" spans="1:4">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>16</v>
       </c>
@@ -6361,7 +6535,7 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="9" spans="1:4">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>16</v>
       </c>
@@ -6375,7 +6549,7 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="10" spans="1:4">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>16</v>
       </c>
@@ -6389,7 +6563,7 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="11" spans="1:4">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>16</v>
       </c>
@@ -6403,7 +6577,7 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="12" spans="1:4">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>16</v>
       </c>
@@ -6417,7 +6591,7 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="13" spans="1:4">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>16</v>
       </c>
@@ -6431,7 +6605,7 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="14" spans="1:4">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>16</v>
       </c>
@@ -6445,7 +6619,7 @@
         <v>29880</v>
       </c>
     </row>
-    <row r="15" spans="1:4">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>16</v>
       </c>
@@ -6459,7 +6633,7 @@
         <v>29260</v>
       </c>
     </row>
-    <row r="16" spans="1:4">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>16</v>
       </c>
@@ -6473,7 +6647,7 @@
         <v>28560</v>
       </c>
     </row>
-    <row r="17" spans="1:4">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>16</v>
       </c>
@@ -6487,7 +6661,7 @@
         <v>27910</v>
       </c>
     </row>
-    <row r="18" spans="1:4">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>16</v>
       </c>
@@ -6501,7 +6675,7 @@
         <v>27260</v>
       </c>
     </row>
-    <row r="19" spans="1:4">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>16</v>
       </c>
@@ -6515,7 +6689,7 @@
         <v>26610</v>
       </c>
     </row>
-    <row r="20" spans="1:4">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>16</v>
       </c>
@@ -6529,7 +6703,7 @@
         <v>25960</v>
       </c>
     </row>
-    <row r="21" spans="1:4">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>16</v>
       </c>
@@ -6543,7 +6717,7 @@
         <v>25310</v>
       </c>
     </row>
-    <row r="22" spans="1:4">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>16</v>
       </c>
@@ -6557,7 +6731,7 @@
         <v>24660</v>
       </c>
     </row>
-    <row r="23" spans="1:4">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>16</v>
       </c>
@@ -6571,7 +6745,7 @@
         <v>24010</v>
       </c>
     </row>
-    <row r="24" spans="1:4">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>16</v>
       </c>
@@ -6585,7 +6759,7 @@
         <v>23360</v>
       </c>
     </row>
-    <row r="25" spans="1:4">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>15</v>
       </c>
@@ -6599,7 +6773,7 @@
         <v>22505</v>
       </c>
     </row>
-    <row r="26" spans="1:4">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>15</v>
       </c>
@@ -6613,7 +6787,7 @@
         <v>22505</v>
       </c>
     </row>
-    <row r="27" spans="1:4">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>15</v>
       </c>
@@ -6627,7 +6801,7 @@
         <v>22505</v>
       </c>
     </row>
-    <row r="28" spans="1:4">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>15</v>
       </c>
@@ -6641,7 +6815,7 @@
         <v>22505</v>
       </c>
     </row>
-    <row r="29" spans="1:4">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>15</v>
       </c>
@@ -6655,7 +6829,7 @@
         <v>22505</v>
       </c>
     </row>
-    <row r="30" spans="1:4">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>15</v>
       </c>
@@ -6669,7 +6843,7 @@
         <v>22505</v>
       </c>
     </row>
-    <row r="31" spans="1:4">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>15</v>
       </c>
@@ -6683,7 +6857,7 @@
         <v>22505</v>
       </c>
     </row>
-    <row r="32" spans="1:4">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>15</v>
       </c>
@@ -6697,7 +6871,7 @@
         <v>22505</v>
       </c>
     </row>
-    <row r="33" spans="1:4">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>15</v>
       </c>
@@ -6711,7 +6885,7 @@
         <v>22505</v>
       </c>
     </row>
-    <row r="34" spans="1:4">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>15</v>
       </c>
@@ -6725,7 +6899,7 @@
         <v>21630</v>
       </c>
     </row>
-    <row r="35" spans="1:4">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>15</v>
       </c>
@@ -6739,7 +6913,7 @@
         <v>20690</v>
       </c>
     </row>
-    <row r="36" spans="1:4">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>15</v>
       </c>
@@ -6753,7 +6927,7 @@
         <v>19165</v>
       </c>
     </row>
-    <row r="37" spans="1:4">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>15</v>
       </c>
@@ -6767,7 +6941,7 @@
         <v>18440</v>
       </c>
     </row>
-    <row r="38" spans="1:4">
+    <row r="38" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>15</v>
       </c>
@@ -6781,7 +6955,7 @@
         <v>17785</v>
       </c>
     </row>
-    <row r="39" spans="1:4">
+    <row r="39" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>15</v>
       </c>
@@ -6795,7 +6969,7 @@
         <v>16115</v>
       </c>
     </row>
-    <row r="40" spans="1:4">
+    <row r="40" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>12</v>
       </c>
@@ -6809,7 +6983,7 @@
         <v>19725</v>
       </c>
     </row>
-    <row r="41" spans="1:4">
+    <row r="41" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>12</v>
       </c>
@@ -6823,7 +6997,7 @@
         <v>19725</v>
       </c>
     </row>
-    <row r="42" spans="1:4">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>12</v>
       </c>
@@ -6837,7 +7011,7 @@
         <v>19725</v>
       </c>
     </row>
-    <row r="43" spans="1:4">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>12</v>
       </c>
@@ -6851,7 +7025,7 @@
         <v>19725</v>
       </c>
     </row>
-    <row r="44" spans="1:4">
+    <row r="44" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>12</v>
       </c>
@@ -6865,7 +7039,7 @@
         <v>19725</v>
       </c>
     </row>
-    <row r="45" spans="1:4">
+    <row r="45" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>12</v>
       </c>
@@ -6879,7 +7053,7 @@
         <v>17750</v>
       </c>
     </row>
-    <row r="46" spans="1:4">
+    <row r="46" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>12</v>
       </c>

</xml_diff>

<commit_message>
adding extra system information to frontend details page
</commit_message>
<xml_diff>
--- a/backend/assets/data/fujitsu_capacities_calculated.xlsx
+++ b/backend/assets/data/fujitsu_capacities_calculated.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://pardigmpartners-my.sharepoint.com/personal/alex_paradigm-esco_com/Documents/data_operations/ashp_calculator/backend/assets/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="26" documentId="13_ncr:1_{D420F103-AC1D-4B35-A441-D57FBF080E0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7573420A-3779-4C44-8361-9FBDA80001B9}"/>
+  <xr:revisionPtr revIDLastSave="34" documentId="13_ncr:1_{D420F103-AC1D-4B35-A441-D57FBF080E0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C634B1E9-07E3-4BC0-A3B4-EFD420E9B3DF}"/>
   <bookViews>
-    <workbookView xWindow="6110" yWindow="820" windowWidth="30890" windowHeight="17460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5690" yWindow="2620" windowWidth="30890" windowHeight="17110" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="indoor_combinations" sheetId="2" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="425" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="433" uniqueCount="35">
   <si>
     <t>Model</t>
   </si>
@@ -119,6 +119,30 @@
   <si>
     <t>AOUH48KUAS1</t>
   </si>
+  <si>
+    <t>Op. Watts/Htg</t>
+  </si>
+  <si>
+    <t>Breaker Req.</t>
+  </si>
+  <si>
+    <t>BTU @ 5*F</t>
+  </si>
+  <si>
+    <t>BTU @ 0*F</t>
+  </si>
+  <si>
+    <t>Tonnage</t>
+  </si>
+  <si>
+    <t>SEER2</t>
+  </si>
+  <si>
+    <t>EER2</t>
+  </si>
+  <si>
+    <t>HSPF2</t>
+  </si>
 </sst>
 </file>
 
@@ -163,13 +187,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -186,6 +210,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -451,7 +479,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2E4304B4-14C5-40DF-85A6-AED3FDED911B}">
-  <dimension ref="A1:N183"/>
+  <dimension ref="A1:U183"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="14.26953125" bestFit="1" customWidth="1"/>
@@ -462,9 +490,16 @@
     <col min="8" max="9" width="17.453125" bestFit="1" customWidth="1"/>
     <col min="10" max="11" width="17.453125" customWidth="1"/>
     <col min="12" max="12" width="12.453125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="12.90625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="11.453125" bestFit="1" customWidth="1"/>
+    <col min="16" max="17" width="9.81640625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="8" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="5.81640625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="4.90625" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="5.90625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -501,8 +536,32 @@
       <c r="L1" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="N1" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" t="s">
+        <v>28</v>
+      </c>
+      <c r="P1" t="s">
+        <v>29</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>30</v>
+      </c>
+      <c r="R1" t="s">
+        <v>31</v>
+      </c>
+      <c r="S1" t="s">
+        <v>32</v>
+      </c>
+      <c r="T1" t="s">
+        <v>33</v>
+      </c>
+      <c r="U1" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="2" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>12</v>
       </c>
@@ -528,7 +587,7 @@
         <v>16335</v>
       </c>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>12</v>
       </c>
@@ -554,7 +613,7 @@
         <v>17750</v>
       </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>12</v>
       </c>
@@ -580,7 +639,7 @@
         <v>19725</v>
       </c>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>12</v>
       </c>
@@ -606,7 +665,7 @@
         <v>19725</v>
       </c>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>12</v>
       </c>
@@ -632,7 +691,7 @@
         <v>19725</v>
       </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>12</v>
       </c>
@@ -658,7 +717,7 @@
         <v>19725</v>
       </c>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>12</v>
       </c>
@@ -684,7 +743,7 @@
         <v>19725</v>
       </c>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>12</v>
       </c>
@@ -710,7 +769,7 @@
         <v>19725</v>
       </c>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>12</v>
       </c>
@@ -736,7 +795,7 @@
         <v>16335</v>
       </c>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>12</v>
       </c>
@@ -762,7 +821,7 @@
         <v>17750</v>
       </c>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>12</v>
       </c>
@@ -788,7 +847,7 @@
         <v>19725</v>
       </c>
     </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>12</v>
       </c>
@@ -814,7 +873,7 @@
         <v>19725</v>
       </c>
     </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>12</v>
       </c>
@@ -840,7 +899,7 @@
         <v>19725</v>
       </c>
     </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>12</v>
       </c>
@@ -866,7 +925,7 @@
         <v>19725</v>
       </c>
     </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>15</v>
       </c>
@@ -6224,7 +6283,7 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="177" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="177" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A177" t="s">
         <v>16</v>
       </c>
@@ -6262,154 +6321,298 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="178" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A178" s="3" t="s">
+    <row r="178" spans="1:21" x14ac:dyDescent="0.35">
+      <c r="A178" s="2" t="s">
         <v>21</v>
       </c>
       <c r="B178" t="s">
         <v>14</v>
       </c>
-      <c r="C178" s="3">
-        <v>12</v>
-      </c>
-      <c r="D178" s="3">
-        <v>12</v>
-      </c>
-      <c r="E178" s="4"/>
-      <c r="F178" s="3"/>
-      <c r="G178" s="3"/>
-      <c r="H178" s="4">
+      <c r="C178" s="2">
+        <v>12</v>
+      </c>
+      <c r="D178" s="2">
+        <v>12</v>
+      </c>
+      <c r="E178" s="3"/>
+      <c r="F178" s="2"/>
+      <c r="G178" s="2"/>
+      <c r="H178" s="3">
         <v>15310</v>
       </c>
-      <c r="I178" s="3"/>
-      <c r="J178" s="3"/>
-      <c r="L178" s="4">
+      <c r="I178" s="2"/>
+      <c r="J178" s="2"/>
+      <c r="L178" s="3">
         <v>15310</v>
       </c>
-    </row>
-    <row r="179" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A179" s="3" t="s">
+      <c r="N178" s="3">
+        <v>3408</v>
+      </c>
+      <c r="O178" s="2">
+        <v>15</v>
+      </c>
+      <c r="P178" s="3">
+        <v>16100</v>
+      </c>
+      <c r="Q178" s="3">
+        <v>15310</v>
+      </c>
+      <c r="R178" s="2">
+        <v>1</v>
+      </c>
+      <c r="S178" s="2">
+        <v>19.899999999999999</v>
+      </c>
+      <c r="T178" s="2">
+        <v>13</v>
+      </c>
+      <c r="U178" s="2">
+        <v>10.3</v>
+      </c>
+    </row>
+    <row r="179" spans="1:21" x14ac:dyDescent="0.35">
+      <c r="A179" s="2" t="s">
         <v>22</v>
       </c>
       <c r="B179" t="s">
         <v>14</v>
       </c>
-      <c r="C179" s="3">
+      <c r="C179" s="2">
         <v>18</v>
       </c>
-      <c r="D179" s="3">
+      <c r="D179" s="2">
         <v>18</v>
       </c>
-      <c r="E179" s="4"/>
-      <c r="F179" s="3"/>
-      <c r="G179" s="3"/>
-      <c r="H179" s="4">
+      <c r="E179" s="3"/>
+      <c r="F179" s="2"/>
+      <c r="G179" s="2"/>
+      <c r="H179" s="3">
         <v>15935</v>
       </c>
-      <c r="I179" s="3"/>
-      <c r="J179" s="3"/>
-      <c r="L179" s="4">
+      <c r="I179" s="2"/>
+      <c r="J179" s="2"/>
+      <c r="L179" s="3">
         <v>15935</v>
       </c>
-    </row>
-    <row r="180" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A180" s="3" t="s">
+      <c r="N179" s="3">
+        <v>3552</v>
+      </c>
+      <c r="O179" s="2">
+        <v>20</v>
+      </c>
+      <c r="P179" s="3">
+        <v>17300</v>
+      </c>
+      <c r="Q179" s="3">
+        <v>15935</v>
+      </c>
+      <c r="R179" s="2">
+        <v>1.5</v>
+      </c>
+      <c r="S179" s="2">
+        <v>19.2</v>
+      </c>
+      <c r="T179" s="2">
+        <v>19.2</v>
+      </c>
+      <c r="U179" s="2">
+        <v>10.5</v>
+      </c>
+    </row>
+    <row r="180" spans="1:21" x14ac:dyDescent="0.35">
+      <c r="A180" s="2" t="s">
         <v>23</v>
       </c>
       <c r="B180" t="s">
         <v>14</v>
       </c>
-      <c r="C180" s="3">
+      <c r="C180" s="2">
         <v>24</v>
       </c>
-      <c r="D180" s="3">
+      <c r="D180" s="2">
         <v>24</v>
       </c>
-      <c r="E180" s="4"/>
-      <c r="F180" s="3"/>
-      <c r="G180" s="3"/>
-      <c r="H180" s="4">
+      <c r="E180" s="3"/>
+      <c r="F180" s="2"/>
+      <c r="G180" s="2"/>
+      <c r="H180" s="3">
         <v>23230</v>
       </c>
-      <c r="I180" s="3"/>
-      <c r="J180" s="3"/>
-      <c r="L180" s="4">
+      <c r="I180" s="2"/>
+      <c r="J180" s="2"/>
+      <c r="L180" s="3">
         <v>23230</v>
       </c>
-    </row>
-    <row r="181" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A181" s="3" t="s">
+      <c r="N180" s="3">
+        <v>3816</v>
+      </c>
+      <c r="O180" s="2">
+        <v>20</v>
+      </c>
+      <c r="P180" s="3">
+        <v>24600</v>
+      </c>
+      <c r="Q180" s="3">
+        <v>23230</v>
+      </c>
+      <c r="R180" s="2">
+        <v>2</v>
+      </c>
+      <c r="S180" s="2">
+        <v>17.7</v>
+      </c>
+      <c r="T180" s="2">
+        <v>11.8</v>
+      </c>
+      <c r="U180" s="2">
+        <v>10.1</v>
+      </c>
+    </row>
+    <row r="181" spans="1:21" x14ac:dyDescent="0.35">
+      <c r="A181" s="2" t="s">
         <v>24</v>
       </c>
       <c r="B181" t="s">
         <v>14</v>
       </c>
-      <c r="C181" s="3">
+      <c r="C181" s="2">
         <v>30</v>
       </c>
-      <c r="D181" s="3">
+      <c r="D181" s="2">
         <v>30</v>
       </c>
-      <c r="E181" s="4"/>
-      <c r="F181" s="3"/>
-      <c r="G181" s="3"/>
-      <c r="H181" s="4">
+      <c r="E181" s="3"/>
+      <c r="F181" s="2"/>
+      <c r="G181" s="2"/>
+      <c r="H181" s="3">
         <v>27295</v>
       </c>
-      <c r="I181" s="3"/>
-      <c r="J181" s="3"/>
-      <c r="L181" s="4">
+      <c r="I181" s="2"/>
+      <c r="J181" s="2"/>
+      <c r="L181" s="3">
         <v>27295</v>
       </c>
-    </row>
-    <row r="182" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A182" s="3" t="s">
+      <c r="N181" s="3">
+        <v>4752</v>
+      </c>
+      <c r="O181" s="2">
         <v>25</v>
       </c>
+      <c r="P181" s="3">
+        <v>29400</v>
+      </c>
+      <c r="Q181" s="3">
+        <v>27295</v>
+      </c>
+      <c r="R181" s="2">
+        <v>2.5</v>
+      </c>
+      <c r="S181" s="2">
+        <v>19</v>
+      </c>
+      <c r="T181" s="2">
+        <v>11.7</v>
+      </c>
+      <c r="U181" s="2">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="182" spans="1:21" x14ac:dyDescent="0.35">
+      <c r="A182" s="2" t="s">
+        <v>25</v>
+      </c>
       <c r="B182" t="s">
         <v>14</v>
       </c>
-      <c r="C182" s="3">
+      <c r="C182" s="2">
         <v>36</v>
       </c>
-      <c r="D182" s="3">
+      <c r="D182" s="2">
         <v>36</v>
       </c>
-      <c r="E182" s="4"/>
-      <c r="F182" s="3"/>
-      <c r="G182" s="3"/>
-      <c r="H182" s="4">
+      <c r="E182" s="3"/>
+      <c r="F182" s="2"/>
+      <c r="G182" s="2"/>
+      <c r="H182" s="3">
         <v>29925</v>
       </c>
-      <c r="I182" s="3"/>
-      <c r="J182" s="3"/>
-      <c r="L182" s="4">
+      <c r="I182" s="2"/>
+      <c r="J182" s="2"/>
+      <c r="L182" s="3">
         <v>29925</v>
       </c>
-    </row>
-    <row r="183" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A183" s="3" t="s">
+      <c r="N182" s="3">
+        <v>4992</v>
+      </c>
+      <c r="O182" s="2">
+        <v>25</v>
+      </c>
+      <c r="P182" s="3">
+        <v>32000</v>
+      </c>
+      <c r="Q182" s="3">
+        <v>29925</v>
+      </c>
+      <c r="R182" s="2">
+        <v>3</v>
+      </c>
+      <c r="S182" s="2">
+        <v>17.600000000000001</v>
+      </c>
+      <c r="T182" s="2">
+        <v>10.6</v>
+      </c>
+      <c r="U182" s="2">
+        <v>9.8000000000000007</v>
+      </c>
+    </row>
+    <row r="183" spans="1:21" x14ac:dyDescent="0.35">
+      <c r="A183" s="2" t="s">
         <v>26</v>
       </c>
       <c r="B183" t="s">
         <v>14</v>
       </c>
-      <c r="C183" s="3">
+      <c r="C183" s="2">
         <v>48</v>
       </c>
-      <c r="D183" s="3">
+      <c r="D183" s="2">
         <v>48</v>
       </c>
-      <c r="E183" s="4"/>
-      <c r="F183" s="3"/>
-      <c r="G183" s="3"/>
-      <c r="H183" s="4">
+      <c r="E183" s="3"/>
+      <c r="F183" s="2"/>
+      <c r="G183" s="2"/>
+      <c r="H183" s="3">
         <v>39480</v>
       </c>
-      <c r="I183" s="3"/>
-      <c r="J183" s="3"/>
-      <c r="L183" s="4">
+      <c r="I183" s="2"/>
+      <c r="J183" s="2"/>
+      <c r="L183" s="3">
         <v>39480</v>
+      </c>
+      <c r="N183" s="3">
+        <v>6000</v>
+      </c>
+      <c r="O183" s="2">
+        <v>30</v>
+      </c>
+      <c r="P183" s="3">
+        <v>41000</v>
+      </c>
+      <c r="Q183" s="3">
+        <v>39480</v>
+      </c>
+      <c r="R183" s="2">
+        <v>3.79</v>
+      </c>
+      <c r="S183" s="2">
+        <v>17</v>
+      </c>
+      <c r="T183" s="2">
+        <v>9.5</v>
+      </c>
+      <c r="U183" s="2">
+        <v>9.6</v>
       </c>
     </row>
   </sheetData>
@@ -6430,12 +6633,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
+      <c r="B1" s="4"/>
+      <c r="C1" s="4"/>
+      <c r="D1" s="4"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">

</xml_diff>

<commit_message>
added new fujitsu models
</commit_message>
<xml_diff>
--- a/backend/assets/data/fujitsu_capacities_calculated.xlsx
+++ b/backend/assets/data/fujitsu_capacities_calculated.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29816"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://pardigmpartners-my.sharepoint.com/personal/alex_paradigm-esco_com/Documents/data_operations/ashp_calculator/backend/assets/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="277" documentId="13_ncr:1_{D420F103-AC1D-4B35-A441-D57FBF080E0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5F283166-8CE5-426D-945D-8A1DD982EAAE}"/>
+  <xr:revisionPtr revIDLastSave="296" documentId="13_ncr:1_{D420F103-AC1D-4B35-A441-D57FBF080E0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{153E2128-3854-43EC-A3FF-472A9CE7E92E}"/>
   <bookViews>
-    <workbookView xWindow="42270" yWindow="1540" windowWidth="33310" windowHeight="17110" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="390" yWindow="1130" windowWidth="14400" windowHeight="8170" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="indoor_combinations" sheetId="2" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="433" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="439" uniqueCount="38">
   <si>
     <t>Model</t>
   </si>
@@ -143,12 +143,21 @@
   <si>
     <t>Capacity at 70F (Btu/h)</t>
   </si>
+  <si>
+    <t>AOUH30KUAH1</t>
+  </si>
+  <si>
+    <t>AOUH36KUAH1</t>
+  </si>
+  <si>
+    <t>AOUH48KUAH1</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -475,28 +484,28 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2E4304B4-14C5-40DF-85A6-AED3FDED911B}">
-  <dimension ref="A1:U183"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <dimension ref="A1:U186"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="14.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.26953125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="14" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="6.28515625" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="5.7109375" customWidth="1"/>
-    <col min="8" max="9" width="17.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="11" width="17.42578125" customWidth="1"/>
-    <col min="12" max="12" width="12.42578125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="11.42578125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="10.85546875" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="6.26953125" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="5.7265625" customWidth="1"/>
+    <col min="8" max="9" width="17.453125" bestFit="1" customWidth="1"/>
+    <col min="10" max="11" width="17.453125" customWidth="1"/>
+    <col min="12" max="12" width="12.453125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="11.453125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="10.81640625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="9.81640625" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="8" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="5.85546875" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="4.85546875" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="5.85546875" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="5.81640625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="4.81640625" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="5.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21">
+    <row r="1" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -558,7 +567,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="2" spans="1:21">
+    <row r="2" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>20</v>
       </c>
@@ -608,7 +617,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:21">
+    <row r="3" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>20</v>
       </c>
@@ -658,7 +667,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:21">
+    <row r="4" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>20</v>
       </c>
@@ -708,7 +717,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:21">
+    <row r="5" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>20</v>
       </c>
@@ -758,7 +767,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="6" spans="1:21">
+    <row r="6" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>20</v>
       </c>
@@ -808,7 +817,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:21">
+    <row r="7" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>20</v>
       </c>
@@ -858,7 +867,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="8" spans="1:21">
+    <row r="8" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>20</v>
       </c>
@@ -908,7 +917,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="9" spans="1:21">
+    <row r="9" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>20</v>
       </c>
@@ -958,7 +967,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="10" spans="1:21">
+    <row r="10" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>20</v>
       </c>
@@ -1008,7 +1017,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="11" spans="1:21">
+    <row r="11" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>20</v>
       </c>
@@ -1058,7 +1067,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="12" spans="1:21">
+    <row r="12" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>20</v>
       </c>
@@ -1108,7 +1117,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:21">
+    <row r="13" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>20</v>
       </c>
@@ -1158,7 +1167,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="14" spans="1:21">
+    <row r="14" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>20</v>
       </c>
@@ -1208,7 +1217,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="15" spans="1:21">
+    <row r="15" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>20</v>
       </c>
@@ -1258,7 +1267,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="16" spans="1:21">
+    <row r="16" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>23</v>
       </c>
@@ -1311,7 +1320,7 @@
         <v>11.5</v>
       </c>
     </row>
-    <row r="17" spans="1:21">
+    <row r="17" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>23</v>
       </c>
@@ -1364,7 +1373,7 @@
         <v>11.5</v>
       </c>
     </row>
-    <row r="18" spans="1:21">
+    <row r="18" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>23</v>
       </c>
@@ -1417,7 +1426,7 @@
         <v>11.5</v>
       </c>
     </row>
-    <row r="19" spans="1:21">
+    <row r="19" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>23</v>
       </c>
@@ -1470,7 +1479,7 @@
         <v>11.5</v>
       </c>
     </row>
-    <row r="20" spans="1:21">
+    <row r="20" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>23</v>
       </c>
@@ -1523,7 +1532,7 @@
         <v>11.5</v>
       </c>
     </row>
-    <row r="21" spans="1:21">
+    <row r="21" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>23</v>
       </c>
@@ -1576,7 +1585,7 @@
         <v>11.5</v>
       </c>
     </row>
-    <row r="22" spans="1:21">
+    <row r="22" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>23</v>
       </c>
@@ -1629,7 +1638,7 @@
         <v>11.5</v>
       </c>
     </row>
-    <row r="23" spans="1:21">
+    <row r="23" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>23</v>
       </c>
@@ -1682,7 +1691,7 @@
         <v>11.5</v>
       </c>
     </row>
-    <row r="24" spans="1:21">
+    <row r="24" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>23</v>
       </c>
@@ -1735,7 +1744,7 @@
         <v>11.5</v>
       </c>
     </row>
-    <row r="25" spans="1:21">
+    <row r="25" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>23</v>
       </c>
@@ -1788,7 +1797,7 @@
         <v>11.5</v>
       </c>
     </row>
-    <row r="26" spans="1:21">
+    <row r="26" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>23</v>
       </c>
@@ -1841,7 +1850,7 @@
         <v>11.5</v>
       </c>
     </row>
-    <row r="27" spans="1:21">
+    <row r="27" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>23</v>
       </c>
@@ -1894,7 +1903,7 @@
         <v>11.5</v>
       </c>
     </row>
-    <row r="28" spans="1:21">
+    <row r="28" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>23</v>
       </c>
@@ -1947,7 +1956,7 @@
         <v>11.5</v>
       </c>
     </row>
-    <row r="29" spans="1:21">
+    <row r="29" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>23</v>
       </c>
@@ -2005,7 +2014,7 @@
         <v>11.5</v>
       </c>
     </row>
-    <row r="30" spans="1:21">
+    <row r="30" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>23</v>
       </c>
@@ -2063,7 +2072,7 @@
         <v>11.5</v>
       </c>
     </row>
-    <row r="31" spans="1:21">
+    <row r="31" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>23</v>
       </c>
@@ -2121,7 +2130,7 @@
         <v>11.5</v>
       </c>
     </row>
-    <row r="32" spans="1:21">
+    <row r="32" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>23</v>
       </c>
@@ -2179,7 +2188,7 @@
         <v>11.5</v>
       </c>
     </row>
-    <row r="33" spans="1:21">
+    <row r="33" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>23</v>
       </c>
@@ -2237,7 +2246,7 @@
         <v>11.5</v>
       </c>
     </row>
-    <row r="34" spans="1:21">
+    <row r="34" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>23</v>
       </c>
@@ -2295,7 +2304,7 @@
         <v>11.5</v>
       </c>
     </row>
-    <row r="35" spans="1:21">
+    <row r="35" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>23</v>
       </c>
@@ -2353,7 +2362,7 @@
         <v>11.5</v>
       </c>
     </row>
-    <row r="36" spans="1:21">
+    <row r="36" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>23</v>
       </c>
@@ -2411,7 +2420,7 @@
         <v>11.5</v>
       </c>
     </row>
-    <row r="37" spans="1:21">
+    <row r="37" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>23</v>
       </c>
@@ -2469,7 +2478,7 @@
         <v>11.5</v>
       </c>
     </row>
-    <row r="38" spans="1:21">
+    <row r="38" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>23</v>
       </c>
@@ -2527,7 +2536,7 @@
         <v>11.5</v>
       </c>
     </row>
-    <row r="39" spans="1:21">
+    <row r="39" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>23</v>
       </c>
@@ -2579,7 +2588,7 @@
         <v>11.5</v>
       </c>
     </row>
-    <row r="40" spans="1:21">
+    <row r="40" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>23</v>
       </c>
@@ -2631,7 +2640,7 @@
         <v>11.5</v>
       </c>
     </row>
-    <row r="41" spans="1:21">
+    <row r="41" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>23</v>
       </c>
@@ -2683,7 +2692,7 @@
         <v>11.5</v>
       </c>
     </row>
-    <row r="42" spans="1:21">
+    <row r="42" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>23</v>
       </c>
@@ -2735,7 +2744,7 @@
         <v>11.5</v>
       </c>
     </row>
-    <row r="43" spans="1:21">
+    <row r="43" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>23</v>
       </c>
@@ -2787,7 +2796,7 @@
         <v>11.5</v>
       </c>
     </row>
-    <row r="44" spans="1:21">
+    <row r="44" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>23</v>
       </c>
@@ -2839,7 +2848,7 @@
         <v>11.5</v>
       </c>
     </row>
-    <row r="45" spans="1:21">
+    <row r="45" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>23</v>
       </c>
@@ -2891,7 +2900,7 @@
         <v>11.5</v>
       </c>
     </row>
-    <row r="46" spans="1:21">
+    <row r="46" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>23</v>
       </c>
@@ -2943,7 +2952,7 @@
         <v>11.5</v>
       </c>
     </row>
-    <row r="47" spans="1:21">
+    <row r="47" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>23</v>
       </c>
@@ -2995,7 +3004,7 @@
         <v>11.5</v>
       </c>
     </row>
-    <row r="48" spans="1:21">
+    <row r="48" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>23</v>
       </c>
@@ -3053,7 +3062,7 @@
         <v>11.5</v>
       </c>
     </row>
-    <row r="49" spans="1:21">
+    <row r="49" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>23</v>
       </c>
@@ -3111,7 +3120,7 @@
         <v>11.5</v>
       </c>
     </row>
-    <row r="50" spans="1:21">
+    <row r="50" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>23</v>
       </c>
@@ -3169,7 +3178,7 @@
         <v>11.5</v>
       </c>
     </row>
-    <row r="51" spans="1:21">
+    <row r="51" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>23</v>
       </c>
@@ -3227,7 +3236,7 @@
         <v>11.5</v>
       </c>
     </row>
-    <row r="52" spans="1:21">
+    <row r="52" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>23</v>
       </c>
@@ -3285,7 +3294,7 @@
         <v>11.5</v>
       </c>
     </row>
-    <row r="53" spans="1:21">
+    <row r="53" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>23</v>
       </c>
@@ -3343,7 +3352,7 @@
         <v>11.5</v>
       </c>
     </row>
-    <row r="54" spans="1:21">
+    <row r="54" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>23</v>
       </c>
@@ -3401,7 +3410,7 @@
         <v>11.5</v>
       </c>
     </row>
-    <row r="55" spans="1:21">
+    <row r="55" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>23</v>
       </c>
@@ -3459,7 +3468,7 @@
         <v>11.5</v>
       </c>
     </row>
-    <row r="56" spans="1:21">
+    <row r="56" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
         <v>24</v>
       </c>
@@ -3509,7 +3518,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="57" spans="1:21">
+    <row r="57" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
         <v>24</v>
       </c>
@@ -3559,7 +3568,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="58" spans="1:21">
+    <row r="58" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
         <v>24</v>
       </c>
@@ -3609,7 +3618,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="59" spans="1:21">
+    <row r="59" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
         <v>24</v>
       </c>
@@ -3659,7 +3668,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="60" spans="1:21">
+    <row r="60" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
         <v>24</v>
       </c>
@@ -3709,7 +3718,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="61" spans="1:21">
+    <row r="61" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
         <v>24</v>
       </c>
@@ -3759,7 +3768,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="62" spans="1:21">
+    <row r="62" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
         <v>24</v>
       </c>
@@ -3809,7 +3818,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="63" spans="1:21">
+    <row r="63" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
         <v>24</v>
       </c>
@@ -3859,7 +3868,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="64" spans="1:21">
+    <row r="64" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
         <v>24</v>
       </c>
@@ -3915,7 +3924,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="65" spans="1:21">
+    <row r="65" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
         <v>24</v>
       </c>
@@ -3971,7 +3980,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="66" spans="1:21">
+    <row r="66" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
         <v>24</v>
       </c>
@@ -4027,7 +4036,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="67" spans="1:21">
+    <row r="67" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
         <v>24</v>
       </c>
@@ -4083,7 +4092,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="68" spans="1:21">
+    <row r="68" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
         <v>24</v>
       </c>
@@ -4139,7 +4148,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="69" spans="1:21">
+    <row r="69" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
         <v>24</v>
       </c>
@@ -4195,7 +4204,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="70" spans="1:21">
+    <row r="70" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
         <v>24</v>
       </c>
@@ -4251,7 +4260,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="71" spans="1:21">
+    <row r="71" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
         <v>24</v>
       </c>
@@ -4307,7 +4316,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="72" spans="1:21">
+    <row r="72" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
         <v>24</v>
       </c>
@@ -4363,7 +4372,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="73" spans="1:21">
+    <row r="73" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
         <v>24</v>
       </c>
@@ -4419,7 +4428,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="74" spans="1:21">
+    <row r="74" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
         <v>24</v>
       </c>
@@ -4475,7 +4484,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="75" spans="1:21">
+    <row r="75" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
         <v>24</v>
       </c>
@@ -4531,7 +4540,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="76" spans="1:21">
+    <row r="76" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
         <v>24</v>
       </c>
@@ -4587,7 +4596,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="77" spans="1:21">
+    <row r="77" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
         <v>24</v>
       </c>
@@ -4643,7 +4652,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="78" spans="1:21">
+    <row r="78" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
         <v>24</v>
       </c>
@@ -4699,7 +4708,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="79" spans="1:21">
+    <row r="79" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
         <v>24</v>
       </c>
@@ -4755,7 +4764,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="80" spans="1:21">
+    <row r="80" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
         <v>24</v>
       </c>
@@ -4811,7 +4820,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="81" spans="1:21">
+    <row r="81" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
         <v>24</v>
       </c>
@@ -4867,7 +4876,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="82" spans="1:21">
+    <row r="82" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
         <v>24</v>
       </c>
@@ -4923,7 +4932,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="83" spans="1:21">
+    <row r="83" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A83" t="s">
         <v>24</v>
       </c>
@@ -4979,7 +4988,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="84" spans="1:21">
+    <row r="84" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A84" t="s">
         <v>24</v>
       </c>
@@ -5035,7 +5044,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="85" spans="1:21">
+    <row r="85" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A85" t="s">
         <v>24</v>
       </c>
@@ -5091,7 +5100,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="86" spans="1:21">
+    <row r="86" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A86" t="s">
         <v>24</v>
       </c>
@@ -5147,7 +5156,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="87" spans="1:21">
+    <row r="87" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A87" t="s">
         <v>24</v>
       </c>
@@ -5203,7 +5212,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="88" spans="1:21">
+    <row r="88" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A88" t="s">
         <v>24</v>
       </c>
@@ -5259,7 +5268,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="89" spans="1:21">
+    <row r="89" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A89" t="s">
         <v>24</v>
       </c>
@@ -5315,7 +5324,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="90" spans="1:21">
+    <row r="90" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A90" t="s">
         <v>24</v>
       </c>
@@ -5371,7 +5380,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="91" spans="1:21">
+    <row r="91" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A91" t="s">
         <v>24</v>
       </c>
@@ -5427,7 +5436,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="92" spans="1:21">
+    <row r="92" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A92" t="s">
         <v>24</v>
       </c>
@@ -5483,7 +5492,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="93" spans="1:21">
+    <row r="93" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A93" t="s">
         <v>24</v>
       </c>
@@ -5539,7 +5548,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="94" spans="1:21">
+    <row r="94" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A94" t="s">
         <v>24</v>
       </c>
@@ -5595,7 +5604,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="95" spans="1:21">
+    <row r="95" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A95" t="s">
         <v>24</v>
       </c>
@@ -5651,7 +5660,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="96" spans="1:21">
+    <row r="96" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A96" t="s">
         <v>24</v>
       </c>
@@ -5707,7 +5716,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="97" spans="1:21">
+    <row r="97" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A97" t="s">
         <v>24</v>
       </c>
@@ -5763,7 +5772,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="98" spans="1:21">
+    <row r="98" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A98" t="s">
         <v>24</v>
       </c>
@@ -5819,7 +5828,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="99" spans="1:21">
+    <row r="99" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A99" t="s">
         <v>24</v>
       </c>
@@ -5881,7 +5890,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="100" spans="1:21">
+    <row r="100" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A100" t="s">
         <v>24</v>
       </c>
@@ -5943,7 +5952,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="101" spans="1:21">
+    <row r="101" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A101" t="s">
         <v>24</v>
       </c>
@@ -6005,7 +6014,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="102" spans="1:21">
+    <row r="102" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A102" t="s">
         <v>24</v>
       </c>
@@ -6067,7 +6076,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="103" spans="1:21">
+    <row r="103" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A103" t="s">
         <v>24</v>
       </c>
@@ -6129,7 +6138,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="104" spans="1:21">
+    <row r="104" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A104" t="s">
         <v>24</v>
       </c>
@@ -6191,7 +6200,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="105" spans="1:21">
+    <row r="105" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A105" t="s">
         <v>24</v>
       </c>
@@ -6253,7 +6262,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="106" spans="1:21">
+    <row r="106" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A106" t="s">
         <v>24</v>
       </c>
@@ -6315,7 +6324,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="107" spans="1:21">
+    <row r="107" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A107" t="s">
         <v>24</v>
       </c>
@@ -6377,7 +6386,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="108" spans="1:21">
+    <row r="108" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A108" t="s">
         <v>24</v>
       </c>
@@ -6439,7 +6448,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="109" spans="1:21">
+    <row r="109" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A109" t="s">
         <v>24</v>
       </c>
@@ -6501,7 +6510,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="110" spans="1:21">
+    <row r="110" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A110" t="s">
         <v>24</v>
       </c>
@@ -6563,7 +6572,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="111" spans="1:21">
+    <row r="111" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A111" t="s">
         <v>24</v>
       </c>
@@ -6625,7 +6634,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="112" spans="1:21">
+    <row r="112" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A112" t="s">
         <v>24</v>
       </c>
@@ -6687,7 +6696,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="113" spans="1:21">
+    <row r="113" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A113" t="s">
         <v>24</v>
       </c>
@@ -6749,7 +6758,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="114" spans="1:21">
+    <row r="114" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A114" t="s">
         <v>24</v>
       </c>
@@ -6811,7 +6820,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="115" spans="1:21">
+    <row r="115" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A115" t="s">
         <v>24</v>
       </c>
@@ -6873,7 +6882,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="116" spans="1:21">
+    <row r="116" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A116" t="s">
         <v>24</v>
       </c>
@@ -6935,7 +6944,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="117" spans="1:21">
+    <row r="117" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A117" t="s">
         <v>24</v>
       </c>
@@ -6997,7 +7006,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="118" spans="1:21">
+    <row r="118" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A118" t="s">
         <v>24</v>
       </c>
@@ -7059,7 +7068,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="119" spans="1:21">
+    <row r="119" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A119" t="s">
         <v>24</v>
       </c>
@@ -7121,7 +7130,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="120" spans="1:21">
+    <row r="120" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A120" t="s">
         <v>24</v>
       </c>
@@ -7183,7 +7192,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="121" spans="1:21">
+    <row r="121" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A121" t="s">
         <v>24</v>
       </c>
@@ -7245,7 +7254,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="122" spans="1:21">
+    <row r="122" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A122" t="s">
         <v>24</v>
       </c>
@@ -7307,7 +7316,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="123" spans="1:21">
+    <row r="123" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A123" t="s">
         <v>24</v>
       </c>
@@ -7369,7 +7378,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="124" spans="1:21">
+    <row r="124" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A124" t="s">
         <v>24</v>
       </c>
@@ -7431,7 +7440,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="125" spans="1:21">
+    <row r="125" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A125" t="s">
         <v>24</v>
       </c>
@@ -7493,7 +7502,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="126" spans="1:21">
+    <row r="126" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A126" t="s">
         <v>24</v>
       </c>
@@ -7555,7 +7564,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="127" spans="1:21">
+    <row r="127" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A127" t="s">
         <v>24</v>
       </c>
@@ -7617,7 +7626,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="128" spans="1:21">
+    <row r="128" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A128" t="s">
         <v>24</v>
       </c>
@@ -7679,7 +7688,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="129" spans="1:21">
+    <row r="129" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A129" t="s">
         <v>24</v>
       </c>
@@ -7741,7 +7750,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="130" spans="1:21">
+    <row r="130" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A130" t="s">
         <v>24</v>
       </c>
@@ -7791,7 +7800,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="131" spans="1:21">
+    <row r="131" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A131" t="s">
         <v>24</v>
       </c>
@@ -7841,7 +7850,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="132" spans="1:21">
+    <row r="132" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A132" t="s">
         <v>24</v>
       </c>
@@ -7891,7 +7900,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="133" spans="1:21">
+    <row r="133" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A133" t="s">
         <v>24</v>
       </c>
@@ -7941,7 +7950,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="134" spans="1:21">
+    <row r="134" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A134" t="s">
         <v>24</v>
       </c>
@@ -7991,7 +8000,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="135" spans="1:21">
+    <row r="135" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A135" t="s">
         <v>24</v>
       </c>
@@ -8041,7 +8050,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="136" spans="1:21">
+    <row r="136" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A136" t="s">
         <v>24</v>
       </c>
@@ -8097,7 +8106,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="137" spans="1:21">
+    <row r="137" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A137" t="s">
         <v>24</v>
       </c>
@@ -8153,7 +8162,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="138" spans="1:21">
+    <row r="138" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A138" t="s">
         <v>24</v>
       </c>
@@ -8209,7 +8218,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="139" spans="1:21">
+    <row r="139" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A139" t="s">
         <v>24</v>
       </c>
@@ -8265,7 +8274,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="140" spans="1:21">
+    <row r="140" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A140" t="s">
         <v>24</v>
       </c>
@@ -8321,7 +8330,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="141" spans="1:21">
+    <row r="141" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A141" t="s">
         <v>24</v>
       </c>
@@ -8377,7 +8386,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="142" spans="1:21">
+    <row r="142" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A142" t="s">
         <v>24</v>
       </c>
@@ -8433,7 +8442,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="143" spans="1:21">
+    <row r="143" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A143" t="s">
         <v>24</v>
       </c>
@@ -8489,7 +8498,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="144" spans="1:21">
+    <row r="144" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A144" t="s">
         <v>24</v>
       </c>
@@ -8545,7 +8554,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="145" spans="1:21">
+    <row r="145" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A145" t="s">
         <v>24</v>
       </c>
@@ -8601,7 +8610,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="146" spans="1:21">
+    <row r="146" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A146" t="s">
         <v>24</v>
       </c>
@@ -8657,7 +8666,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="147" spans="1:21">
+    <row r="147" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A147" t="s">
         <v>24</v>
       </c>
@@ -8713,7 +8722,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="148" spans="1:21">
+    <row r="148" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A148" t="s">
         <v>24</v>
       </c>
@@ -8769,7 +8778,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="149" spans="1:21">
+    <row r="149" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A149" t="s">
         <v>24</v>
       </c>
@@ -8825,7 +8834,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="150" spans="1:21">
+    <row r="150" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A150" t="s">
         <v>24</v>
       </c>
@@ -8881,7 +8890,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="151" spans="1:21">
+    <row r="151" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A151" t="s">
         <v>24</v>
       </c>
@@ -8937,7 +8946,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="152" spans="1:21">
+    <row r="152" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A152" t="s">
         <v>24</v>
       </c>
@@ -8993,7 +9002,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="153" spans="1:21">
+    <row r="153" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A153" t="s">
         <v>24</v>
       </c>
@@ -9049,7 +9058,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="154" spans="1:21">
+    <row r="154" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A154" t="s">
         <v>24</v>
       </c>
@@ -9105,7 +9114,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="155" spans="1:21">
+    <row r="155" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A155" t="s">
         <v>24</v>
       </c>
@@ -9161,7 +9170,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="156" spans="1:21">
+    <row r="156" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A156" t="s">
         <v>24</v>
       </c>
@@ -9217,7 +9226,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="157" spans="1:21">
+    <row r="157" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A157" t="s">
         <v>24</v>
       </c>
@@ -9279,7 +9288,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="158" spans="1:21">
+    <row r="158" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A158" t="s">
         <v>24</v>
       </c>
@@ -9341,7 +9350,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="159" spans="1:21">
+    <row r="159" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A159" t="s">
         <v>24</v>
       </c>
@@ -9403,7 +9412,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="160" spans="1:21">
+    <row r="160" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A160" t="s">
         <v>24</v>
       </c>
@@ -9465,7 +9474,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="161" spans="1:21">
+    <row r="161" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A161" t="s">
         <v>24</v>
       </c>
@@ -9527,7 +9536,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="162" spans="1:21">
+    <row r="162" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A162" t="s">
         <v>24</v>
       </c>
@@ -9589,7 +9598,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="163" spans="1:21">
+    <row r="163" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A163" t="s">
         <v>24</v>
       </c>
@@ -9651,7 +9660,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="164" spans="1:21">
+    <row r="164" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A164" t="s">
         <v>24</v>
       </c>
@@ -9713,7 +9722,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="165" spans="1:21">
+    <row r="165" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A165" t="s">
         <v>24</v>
       </c>
@@ -9775,7 +9784,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="166" spans="1:21">
+    <row r="166" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A166" t="s">
         <v>24</v>
       </c>
@@ -9837,7 +9846,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="167" spans="1:21">
+    <row r="167" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A167" t="s">
         <v>24</v>
       </c>
@@ -9899,7 +9908,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="168" spans="1:21">
+    <row r="168" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A168" t="s">
         <v>24</v>
       </c>
@@ -9961,7 +9970,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="169" spans="1:21">
+    <row r="169" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A169" t="s">
         <v>24</v>
       </c>
@@ -10023,7 +10032,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="170" spans="1:21">
+    <row r="170" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A170" t="s">
         <v>24</v>
       </c>
@@ -10085,7 +10094,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="171" spans="1:21">
+    <row r="171" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A171" t="s">
         <v>24</v>
       </c>
@@ -10147,7 +10156,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="172" spans="1:21">
+    <row r="172" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A172" t="s">
         <v>24</v>
       </c>
@@ -10209,7 +10218,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="173" spans="1:21">
+    <row r="173" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A173" t="s">
         <v>24</v>
       </c>
@@ -10271,7 +10280,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="174" spans="1:21">
+    <row r="174" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A174" t="s">
         <v>24</v>
       </c>
@@ -10333,7 +10342,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="175" spans="1:21">
+    <row r="175" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A175" t="s">
         <v>24</v>
       </c>
@@ -10395,7 +10404,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="176" spans="1:21">
+    <row r="176" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A176" t="s">
         <v>24</v>
       </c>
@@ -10457,7 +10466,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="177" spans="1:21">
+    <row r="177" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A177" t="s">
         <v>24</v>
       </c>
@@ -10519,7 +10528,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="178" spans="1:21">
+    <row r="178" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A178" s="2" t="s">
         <v>25</v>
       </c>
@@ -10568,7 +10577,7 @@
         <v>10.3</v>
       </c>
     </row>
-    <row r="179" spans="1:21">
+    <row r="179" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A179" s="2" t="s">
         <v>26</v>
       </c>
@@ -10617,7 +10626,7 @@
         <v>10.5</v>
       </c>
     </row>
-    <row r="180" spans="1:21">
+    <row r="180" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A180" s="2" t="s">
         <v>27</v>
       </c>
@@ -10666,7 +10675,7 @@
         <v>10.1</v>
       </c>
     </row>
-    <row r="181" spans="1:21">
+    <row r="181" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A181" s="2" t="s">
         <v>28</v>
       </c>
@@ -10715,7 +10724,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="182" spans="1:21">
+    <row r="182" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A182" s="2" t="s">
         <v>29</v>
       </c>
@@ -10764,7 +10773,7 @@
         <v>9.8000000000000007</v>
       </c>
     </row>
-    <row r="183" spans="1:21">
+    <row r="183" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A183" s="2" t="s">
         <v>30</v>
       </c>
@@ -10811,6 +10820,138 @@
       </c>
       <c r="U183" s="2">
         <v>9.6</v>
+      </c>
+    </row>
+    <row r="184" spans="1:21" x14ac:dyDescent="0.35">
+      <c r="A184" t="s">
+        <v>35</v>
+      </c>
+      <c r="B184" t="s">
+        <v>22</v>
+      </c>
+      <c r="C184" s="2">
+        <v>30</v>
+      </c>
+      <c r="D184" s="2">
+        <v>30</v>
+      </c>
+      <c r="H184" s="3">
+        <v>31940</v>
+      </c>
+      <c r="L184" s="3">
+        <v>31940</v>
+      </c>
+      <c r="N184" s="3">
+        <v>6432</v>
+      </c>
+      <c r="O184" s="2">
+        <v>30</v>
+      </c>
+      <c r="P184" s="3">
+        <v>34000</v>
+      </c>
+      <c r="Q184" s="3">
+        <v>31940</v>
+      </c>
+      <c r="R184" s="2">
+        <v>2.5</v>
+      </c>
+      <c r="S184" s="2">
+        <v>18.8</v>
+      </c>
+      <c r="T184" s="2">
+        <v>12.2</v>
+      </c>
+      <c r="U184" s="2">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="185" spans="1:21" x14ac:dyDescent="0.35">
+      <c r="A185" t="s">
+        <v>36</v>
+      </c>
+      <c r="B185" t="s">
+        <v>22</v>
+      </c>
+      <c r="C185" s="2">
+        <v>36</v>
+      </c>
+      <c r="D185" s="2">
+        <v>36</v>
+      </c>
+      <c r="H185" s="3">
+        <v>38750</v>
+      </c>
+      <c r="L185" s="3">
+        <v>38750</v>
+      </c>
+      <c r="N185" s="3">
+        <v>6720</v>
+      </c>
+      <c r="O185" s="2">
+        <v>35</v>
+      </c>
+      <c r="P185" s="3">
+        <v>41000</v>
+      </c>
+      <c r="Q185" s="3">
+        <v>38750</v>
+      </c>
+      <c r="R185" s="2">
+        <v>3</v>
+      </c>
+      <c r="S185" s="2">
+        <v>18.3</v>
+      </c>
+      <c r="T185" s="2">
+        <v>11.4</v>
+      </c>
+      <c r="U185" s="2">
+        <v>10.199999999999999</v>
+      </c>
+    </row>
+    <row r="186" spans="1:21" x14ac:dyDescent="0.35">
+      <c r="A186" t="s">
+        <v>37</v>
+      </c>
+      <c r="B186" t="s">
+        <v>22</v>
+      </c>
+      <c r="C186" s="2">
+        <v>48</v>
+      </c>
+      <c r="D186" s="2">
+        <v>48</v>
+      </c>
+      <c r="H186" s="3">
+        <v>48000</v>
+      </c>
+      <c r="L186" s="3">
+        <v>48000</v>
+      </c>
+      <c r="N186" s="3">
+        <v>8904</v>
+      </c>
+      <c r="O186" s="2">
+        <v>45</v>
+      </c>
+      <c r="P186" s="3">
+        <v>51000</v>
+      </c>
+      <c r="Q186" s="3">
+        <v>48000</v>
+      </c>
+      <c r="R186" s="2">
+        <v>3.79</v>
+      </c>
+      <c r="S186" s="2">
+        <v>19</v>
+      </c>
+      <c r="T186" s="2">
+        <v>11.2</v>
+      </c>
+      <c r="U186" s="2">
+        <v>10.199999999999999</v>
       </c>
     </row>
   </sheetData>
@@ -10822,15 +10963,15 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D46"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="15.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="21.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.26953125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.453125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" s="4" t="s">
         <v>31</v>
       </c>
@@ -10838,7 +10979,7 @@
       <c r="C1" s="4"/>
       <c r="D1" s="4"/>
     </row>
-    <row r="2" spans="1:4">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -10852,7 +10993,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="3" spans="1:4">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>24</v>
       </c>
@@ -10866,7 +11007,7 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="4" spans="1:4">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>24</v>
       </c>
@@ -10880,7 +11021,7 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="5" spans="1:4">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>24</v>
       </c>
@@ -10894,7 +11035,7 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="6" spans="1:4">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>24</v>
       </c>
@@ -10908,7 +11049,7 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="7" spans="1:4">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>24</v>
       </c>
@@ -10922,7 +11063,7 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="8" spans="1:4">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>24</v>
       </c>
@@ -10936,7 +11077,7 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="9" spans="1:4">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>24</v>
       </c>
@@ -10950,7 +11091,7 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="10" spans="1:4">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>24</v>
       </c>
@@ -10964,7 +11105,7 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="11" spans="1:4">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>24</v>
       </c>
@@ -10978,7 +11119,7 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="12" spans="1:4">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>24</v>
       </c>
@@ -10992,7 +11133,7 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="13" spans="1:4">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>24</v>
       </c>
@@ -11006,7 +11147,7 @@
         <v>30760</v>
       </c>
     </row>
-    <row r="14" spans="1:4">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>24</v>
       </c>
@@ -11020,7 +11161,7 @@
         <v>29880</v>
       </c>
     </row>
-    <row r="15" spans="1:4">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>24</v>
       </c>
@@ -11034,7 +11175,7 @@
         <v>29260</v>
       </c>
     </row>
-    <row r="16" spans="1:4">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>24</v>
       </c>
@@ -11048,7 +11189,7 @@
         <v>28560</v>
       </c>
     </row>
-    <row r="17" spans="1:4">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>24</v>
       </c>
@@ -11062,7 +11203,7 @@
         <v>27910</v>
       </c>
     </row>
-    <row r="18" spans="1:4">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>24</v>
       </c>
@@ -11076,7 +11217,7 @@
         <v>27260</v>
       </c>
     </row>
-    <row r="19" spans="1:4">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>24</v>
       </c>
@@ -11090,7 +11231,7 @@
         <v>26610</v>
       </c>
     </row>
-    <row r="20" spans="1:4">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>24</v>
       </c>
@@ -11104,7 +11245,7 @@
         <v>25960</v>
       </c>
     </row>
-    <row r="21" spans="1:4">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>24</v>
       </c>
@@ -11118,7 +11259,7 @@
         <v>25310</v>
       </c>
     </row>
-    <row r="22" spans="1:4">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>24</v>
       </c>
@@ -11132,7 +11273,7 @@
         <v>24660</v>
       </c>
     </row>
-    <row r="23" spans="1:4">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>24</v>
       </c>
@@ -11146,7 +11287,7 @@
         <v>24010</v>
       </c>
     </row>
-    <row r="24" spans="1:4">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>24</v>
       </c>
@@ -11160,7 +11301,7 @@
         <v>23360</v>
       </c>
     </row>
-    <row r="25" spans="1:4">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>23</v>
       </c>
@@ -11174,7 +11315,7 @@
         <v>22505</v>
       </c>
     </row>
-    <row r="26" spans="1:4">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>23</v>
       </c>
@@ -11188,7 +11329,7 @@
         <v>22505</v>
       </c>
     </row>
-    <row r="27" spans="1:4">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>23</v>
       </c>
@@ -11202,7 +11343,7 @@
         <v>22505</v>
       </c>
     </row>
-    <row r="28" spans="1:4">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>23</v>
       </c>
@@ -11216,7 +11357,7 @@
         <v>22505</v>
       </c>
     </row>
-    <row r="29" spans="1:4">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>23</v>
       </c>
@@ -11230,7 +11371,7 @@
         <v>22505</v>
       </c>
     </row>
-    <row r="30" spans="1:4">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>23</v>
       </c>
@@ -11244,7 +11385,7 @@
         <v>22505</v>
       </c>
     </row>
-    <row r="31" spans="1:4">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>23</v>
       </c>
@@ -11258,7 +11399,7 @@
         <v>22505</v>
       </c>
     </row>
-    <row r="32" spans="1:4">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>23</v>
       </c>
@@ -11272,7 +11413,7 @@
         <v>22505</v>
       </c>
     </row>
-    <row r="33" spans="1:4">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>23</v>
       </c>
@@ -11286,7 +11427,7 @@
         <v>22505</v>
       </c>
     </row>
-    <row r="34" spans="1:4">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>23</v>
       </c>
@@ -11300,7 +11441,7 @@
         <v>21630</v>
       </c>
     </row>
-    <row r="35" spans="1:4">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>23</v>
       </c>
@@ -11314,7 +11455,7 @@
         <v>20690</v>
       </c>
     </row>
-    <row r="36" spans="1:4">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>23</v>
       </c>
@@ -11328,7 +11469,7 @@
         <v>19165</v>
       </c>
     </row>
-    <row r="37" spans="1:4">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>23</v>
       </c>
@@ -11342,7 +11483,7 @@
         <v>18440</v>
       </c>
     </row>
-    <row r="38" spans="1:4">
+    <row r="38" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>23</v>
       </c>
@@ -11356,7 +11497,7 @@
         <v>17785</v>
       </c>
     </row>
-    <row r="39" spans="1:4">
+    <row r="39" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>23</v>
       </c>
@@ -11370,7 +11511,7 @@
         <v>16115</v>
       </c>
     </row>
-    <row r="40" spans="1:4">
+    <row r="40" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>20</v>
       </c>
@@ -11384,7 +11525,7 @@
         <v>19725</v>
       </c>
     </row>
-    <row r="41" spans="1:4">
+    <row r="41" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>20</v>
       </c>
@@ -11398,7 +11539,7 @@
         <v>19725</v>
       </c>
     </row>
-    <row r="42" spans="1:4">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>20</v>
       </c>
@@ -11412,7 +11553,7 @@
         <v>19725</v>
       </c>
     </row>
-    <row r="43" spans="1:4">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>20</v>
       </c>
@@ -11426,7 +11567,7 @@
         <v>19725</v>
       </c>
     </row>
-    <row r="44" spans="1:4">
+    <row r="44" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>20</v>
       </c>
@@ -11440,7 +11581,7 @@
         <v>19725</v>
       </c>
     </row>
-    <row r="45" spans="1:4">
+    <row r="45" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>20</v>
       </c>
@@ -11454,7 +11595,7 @@
         <v>17750</v>
       </c>
     </row>
-    <row r="46" spans="1:4">
+    <row r="46" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>20</v>
       </c>

</xml_diff>

<commit_message>
remove setdetailstext and use detailstext memo
</commit_message>
<xml_diff>
--- a/backend/assets/data/fujitsu_capacities_calculated.xlsx
+++ b/backend/assets/data/fujitsu_capacities_calculated.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://pardigmpartners-my.sharepoint.com/personal/alex_paradigm-esco_com/Documents/data_operations/ashp_calculator/backend/assets/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="296" documentId="13_ncr:1_{D420F103-AC1D-4B35-A441-D57FBF080E0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{153E2128-3854-43EC-A3FF-472A9CE7E92E}"/>
+  <xr:revisionPtr revIDLastSave="302" documentId="13_ncr:1_{D420F103-AC1D-4B35-A441-D57FBF080E0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E29A19E0-3F0A-499A-8CA7-95FE708198C1}"/>
   <bookViews>
-    <workbookView xWindow="390" yWindow="1130" windowWidth="14400" windowHeight="8170" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="41780" yWindow="320" windowWidth="30890" windowHeight="17110" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="indoor_combinations" sheetId="2" r:id="rId1"/>

</xml_diff>